<commit_message>
Add Bangladesh national scale health data expansion and validation
</commit_message>
<xml_diff>
--- a/health_data.xlsx
+++ b/health_data.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health" sheetId="8" r:id="R8a9367a9111e4ebc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health_Catalog_Clean" sheetId="9" r:id="R4dd0025c639249e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health" sheetId="8" r:id="Re6c85285bee54932"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health_Catalog_Clean" sheetId="9" r:id="Rb08629cd6dd64ba1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1086,7 +1086,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="111">
+  <x:cellXfs count="112">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1377,6 +1377,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -3597,20 +3600,95 @@
       <x:c r="AY113" s="3"/>
       <x:c r="AZ113" s="3"/>
     </x:row>
-    <x:row r="114">
-      <x:c r="D114" s="12"/>
-    </x:row>
-    <x:row r="115">
-      <x:c r="D115" s="12"/>
-    </x:row>
-    <x:row r="116">
-      <x:c r="D116" s="12"/>
-    </x:row>
-    <x:row r="117">
-      <x:c r="D117" s="12"/>
-    </x:row>
-    <x:row r="118">
-      <x:c r="D118" s="12"/>
+    <x:row r="114" ht="96" customHeight="1">
+      <x:c r="A114" s="107"/>
+      <x:c r="B114" s="107" t="str">
+        <x:v>DGHS / MoHFW</x:v>
+      </x:c>
+      <x:c r="C114" s="107" t="str">
+        <x:v>Facility and Laboratory Registry</x:v>
+      </x:c>
+      <x:c r="D114" s="111" t="str">
+        <x:v>DGHS Active Facility Registry (Bangladesh)</x:v>
+      </x:c>
+      <x:c r="E114" s="107" t="str">
+        <x:v>https://hrm.dghs.gov.bd/public/facility-registry/reports/organization-list?is_active=1&amp;submit=Run&amp;columns_csv=id%2Cname%2Cname_bn%2Ccode%2Cemail_1%2Cfacility_agency_name%2Cfacility_type_name%2Cdivision_name%2Cdistrict_name%2Ccity_corporation_name%2Cupazila_name%2Cpaurasava_name%2Cunion_name%2Cis_private&amp;alias_columns_csv=ID%2CName%2CName+%28Bangla%29%2CCode%2CEmail%2CAgency%2CType%2CDivision%2CDistrict%2CCity+Corporation%2CUpazila%2CPaurasava%2CUnion%2CPrivate&amp;ret=excel</x:v>
+      </x:c>
+      <x:c r="F114" s="107" t="str">
+        <x:v>XLSX</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="54" customHeight="1">
+      <x:c r="A115" s="107"/>
+      <x:c r="B115" s="107" t="str">
+        <x:v>DGHS / MoHFW</x:v>
+      </x:c>
+      <x:c r="C115" s="107" t="str">
+        <x:v>National Health Interoperability</x:v>
+      </x:c>
+      <x:c r="D115" s="111" t="str">
+        <x:v>Bangladesh Core FHIR Implementation Guide v0.4.6 — Full Package</x:v>
+      </x:c>
+      <x:c r="E115" s="107" t="str">
+        <x:v>https://fhir.dghs.gov.bd/core/full-ig.zip</x:v>
+      </x:c>
+      <x:c r="F115" s="107" t="str">
+        <x:v>ZIP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="54" customHeight="1">
+      <x:c r="A116" s="107"/>
+      <x:c r="B116" s="107" t="str">
+        <x:v>DGHS / MoHFW</x:v>
+      </x:c>
+      <x:c r="C116" s="107" t="str">
+        <x:v>Disease Terminology</x:v>
+      </x:c>
+      <x:c r="D116" s="111" t="str">
+        <x:v>Bangladesh ICD-11 MMS Condition ValueSet (Diagnosis and Finding)</x:v>
+      </x:c>
+      <x:c r="E116" s="107" t="str">
+        <x:v>https://tr.ocl.dghs.gov.bd/api/orgs/MoHFW/collections/bd-condition-icd11-diagnosis-valueset/HEAD/expansions/autoexpand-HEAD/concepts/?limit=1000</x:v>
+      </x:c>
+      <x:c r="F116" s="107" t="str">
+        <x:v>JSON API</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="54" customHeight="1">
+      <x:c r="A117" s="107"/>
+      <x:c r="B117" s="107" t="str">
+        <x:v>DGHS / MoHFW</x:v>
+      </x:c>
+      <x:c r="C117" s="107" t="str">
+        <x:v>Vaccination</x:v>
+      </x:c>
+      <x:c r="D117" s="111" t="str">
+        <x:v>Bangladesh Vaccine Value Set</x:v>
+      </x:c>
+      <x:c r="E117" s="107" t="str">
+        <x:v>https://fhir.dghs.gov.bd/core/ValueSet-bd-vaccine-valueset.html</x:v>
+      </x:c>
+      <x:c r="F117" s="107" t="str">
+        <x:v>HTML/JSON</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="54" customHeight="1">
+      <x:c r="A118" s="107"/>
+      <x:c r="B118" s="107" t="str">
+        <x:v>Bangladesh Open Data</x:v>
+      </x:c>
+      <x:c r="C118" s="107" t="str">
+        <x:v>Health Workforce</x:v>
+      </x:c>
+      <x:c r="D118" s="111" t="str">
+        <x:v>Doctor Directory</x:v>
+      </x:c>
+      <x:c r="E118" s="107" t="str">
+        <x:v>https://data.gov.bd/sites/default/files/data-resource/2016/10/18/Doctor-Directory.xls</x:v>
+      </x:c>
+      <x:c r="F118" s="107" t="str">
+        <x:v>XLS</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="D119" s="12"/>
@@ -3875,121 +3953,121 @@
     <x:mergeCell ref="C46:C73"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="Rc98dc4499651443c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="Rebb19a14808b47da"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="R7c397d99d4d649c5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="R3f168dccf28f489d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="R6a108628d56e429b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="R388974f27a124bbf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="Rc32a3397b80e4845"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="R42458255db3b484d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="Rf6818ace2cd949e4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="R683313ec184c4552"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="R4258edccda904459"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="R756418f1be254835"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="Rab49616679dc4f2c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="R1e0b03fd15a54c32"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R94671e33bd044243"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="R02a0ec93ae814026"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="R0c50c3308cb040a9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="R8daa4b7577854fbf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="Rddd1fdf448904888"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="R09739f80faab4f00"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="Ra90b45e9cfc546b8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="Rc8231bfffc474470"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="R6116149218da4b41"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="Rf5f4189a560b48f2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="Rc25e1592b53f4491"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="Re631bea40f8548bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="R32a4212339284541"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="Rf88774d78f66411f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="Rf8299946d8a8486b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="R4854c23295034e34"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="R5f6e9e44692f43c1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="Rf0199cafee174685"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R9046470ff6474ab2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="R2881d232c5bc478c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="Rf19a474063004af0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="R0797afd8993d4ac8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="Rd070fd17569f4ea2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="Rdf0ff639adb44778"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R999ccb1707184ecb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R2099da1544424fbb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="Ra46c80b5e84f4de7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="Rd9fa2140ccd04266"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Rb438db95c26d4410"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="R4cfa4342dbe94b62"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="Re4cfe6d611754708"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="Rd9a1d8eb04cb4b00"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="R6c8dc321330949c4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="Rcb038009bc4e4c13"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="R939f36a65c784998"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="R0d774cbc7a014993"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R7d42d3fc3c3a4bdb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="Ra9487b55b135467a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="Ra98aec93694c4e0a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="Rd90e047ebfa2432c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="Rf2adbeddf3d04b87"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="R1fb6dd213ead4d6a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="Raee561dab3564b00"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="Rbb933371f4be426e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="R11dab97054b5420a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="R038b60cc50894e01"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="Rc19fcdbf19224eea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R2a999a28b9b14888"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R1972b248199943df"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="R1a5ecb25e7b347a6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="Rc00f429a2bc84dec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="Rb4eac7c5c9e5428c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="Ra3ede4e7e4b748c2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="R0af4e8600b4c49ba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="R6db05b1db28f4aaf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="Ra9712e25b3954f30"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="R344e529974214b27"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="Rf93ac67e828d4688"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="Rcda2a44cc1c1453a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="Rf78a511612c34c5a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="Rb70bd76a1ced4521"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="Rf4e79bedbe474096"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="R40af6d8e1c6f48b1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="Rd3a0703505dc4826"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="R489b7d66b18143a9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="R35d08f53d4d24837"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="R8cc6296cdb9044ae"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="R16aceff8dcb549ec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="Rfdc0831c5a944826"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="R83b5fbb9c9524e61"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="R9f20f2231ea548d7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="Rba2883f666044feb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="R6ea36e301acc4d05"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="R92515fcb3ccb4fe8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="Rc91e375fdc9b4f02"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="R7ef0278b085d4426"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="R16a00e8c3c454ca5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="Rd2df3a353e3a4504"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="R8180fbdbffc74fde"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="R0fc7371f02b74aa0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="R3ef073d26d8847e4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="R9d156da994d24e05"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="R029a64bff1f64864"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="R0706a7bb60c14912"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="Ree14a103326f4c74"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="R57ee42349e32422c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="Rc1044ed12c574171"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="R88c939bdc257403c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="R188fc5abc4704a37"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="R1e354334b35548a4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="Rdac2f6473a904d6b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="Rd8f725551d4d4dc5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="Rae00be92eba64d56"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="R406b31e7a1cc4b7b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="R4d5a88695a994c14"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="R75a53fb9b66f464a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="Rf7dba2db5a6641aa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="R71366b7c9fe947ef"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="R1f7f4de9955d40c2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="Rf3888e2a9136424b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="R46c1f6d8aae54ea3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="R36ddba68a1f04fe1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="R4e7a14adfdb14668"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="R90ab7d3a8cf04880"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="R79995dcaa27e4a7c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="R793ef01277f8472a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="R6505d1c87e6b42a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="R665346b961c84809"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="R45c394ee2cc242fd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="Rb3cc8326818646d9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="Re94a9515ae274edc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="Re1dbf4db9a604481"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="R813df0a08cc1431c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="R4b5f9cb847e94210"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="Rdecdb73b19284c69"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="Rd56d296a350d4d3d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="Ra50138f25f6241d9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="R7f98fbc72f3a4a29"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="Rf3eb8187664c4fd3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="R8749f284a79242c1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="Rce7244587f9b4bd7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="R3e8a65b64e6c42c8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="Rd489d7ab263e47e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="Ra2f9b2b84e124453"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="R4d5989604c97481b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="Rc86ae9da22fa4f12"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="R749dbbe8a302465e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="R5570de8f0c9b4966"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="R7bdbcb9c364443ae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="R4710309807a94b66"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="R49590d20cc7c4a36"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="R12ed0e47d2624fe4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="R8c49a1d9f4644f07"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R7de31df136a143b6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="R71944336d7774d46"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="R859c4636b1e748dc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="R06ff2ed70d54485a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="Re074c1ab40584bcb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="Rabf54c231cc54815"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R8958b702c8044c31"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rc980cabc6f394253"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="Rd3f4207fbe094f84"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="R6294ef5eb7a0406f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Rbd43c50f79b54204"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="R1785cf1ef51c4d63"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="Rd2642835bd594f99"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="R283f7fb16baa4a1d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="Rdf2eedd3892b4311"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="R849809ff01514dde"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="Rcf6cca5986314771"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="Race942c77f254553"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R0b8a8283bf2546c0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R1fd0cba662f04a2b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="Rd03b368863b944ba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="R1df572a66233492c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="R846ac1d639d2438e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="Raae4ced769074d5a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R82af723d29874815"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="Rd0dcc5722e8d480e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="Ra44203f3f5164aa7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="Rd531f6d9a57e432b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="Rc0fca617cfde4bbe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R5207eb9f364247c0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R646247e510ba4f70"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="Rfc4550a2437f490d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="Rc8ff2aa94f644a68"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R95ebe06dcfa04742"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="Rc49bba91a80b44e1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="Rf7a254356a76403c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="R440d256b219b471e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="Rba123870283e4002"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="R7af6d91f4fd94e87"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="R418738121aee4f30"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="Rc405e02e810c4a8b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="R48a151732c014d41"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="Rb97f864d4c3b48de"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="R324b64de71b842a6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="R60860006ab95451b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="Rc23473f7d13648f5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="R29147ab062c6474c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="R17f0684390164683"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="R99377a2c4d444008"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="R62a75d42c59b4465"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="Rd19dd137b8264a1c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="Rc58bf10ae50f4871"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="Rfa7eb017486248a8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="R960de8a0500a420f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="Reb66f06851d042a0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="Rc8d113c17e9140ae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="R0b2f8914f328405a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="Rdf16254457e54898"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="Rf67cea24d2f841f4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="R473e419ac01440fe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="Rfa876d1701644633"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="R3f65a3b016764a3a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="R005fb229c9c64059"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="Re030a500411c419d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="R8a2fe413b83042cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="R1fb8cd498b34499a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="Rb0b88fc334084ee2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="R74f4e4bfc10b4ba8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="R7c58925147644329"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="R94d740552e094563"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="R5c46acfa95144c4f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="R9d7c6aa6a5b140cb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="R7381b6698c9441f8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="R46b57811d2b64e69"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="Rd53defb9c6d54e58"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="R62ad20ccbec748b9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="Ra288e2f6d4274a0e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="Re848affd58954c3d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="Rfe5a752fa5244c38"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="R8a205ef2daff499f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="R1bd3e490e6cf42ad"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="R38d96ff035db472e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="R3be718fc31cf4aae"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6947,10 +7025,140 @@
         <x:v>Primary source entry</x:v>
       </x:c>
     </x:row>
+    <x:row r="114" ht="132" customHeight="1">
+      <x:c r="A114" s="107" t="n">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="B114" s="107" t="str">
+        <x:v>Health</x:v>
+      </x:c>
+      <x:c r="C114" s="107" t="str">
+        <x:v>DGHS / MoHFW</x:v>
+      </x:c>
+      <x:c r="D114" s="107" t="str">
+        <x:v>Facility and Laboratory Registry</x:v>
+      </x:c>
+      <x:c r="E114" s="107" t="str">
+        <x:v>DGHS Active Facility Registry (Bangladesh)</x:v>
+      </x:c>
+      <x:c r="F114" s="107" t="str">
+        <x:v>https://hrm.dghs.gov.bd/public/facility-registry/reports/organization-list?is_active=1&amp;submit=Run&amp;columns_csv=id%2Cname%2Cname_bn%2Ccode%2Cemail_1%2Cfacility_agency_name%2Cfacility_type_name%2Cdivision_name%2Cdistrict_name%2Ccity_corporation_name%2Cupazila_name%2Cpaurasava_name%2Cunion_name%2Cis_private&amp;alias_columns_csv=ID%2CName%2CName+%28Bangla%29%2CCode%2CEmail%2CAgency%2CType%2CDivision%2CDistrict%2CCity+Corporation%2CUpazila%2CPaurasava%2CUnion%2CPrivate&amp;ret=excel</x:v>
+      </x:c>
+      <x:c r="G114" s="107" t="str">
+        <x:v>XLSX dataset</x:v>
+      </x:c>
+      <x:c r="H114" s="107" t="str">
+        <x:v>Official active-facility export; 39,434 complete rows map to HealthFacility and 9,694 diagnostic/laboratory-type rows map to Laboratory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="84" customHeight="1">
+      <x:c r="A115" s="107" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="B115" s="107" t="str">
+        <x:v>Health</x:v>
+      </x:c>
+      <x:c r="C115" s="107" t="str">
+        <x:v>DGHS / MoHFW</x:v>
+      </x:c>
+      <x:c r="D115" s="107" t="str">
+        <x:v>National Health Interoperability</x:v>
+      </x:c>
+      <x:c r="E115" s="107" t="str">
+        <x:v>Bangladesh Core FHIR Implementation Guide v0.4.6 — Full Package</x:v>
+      </x:c>
+      <x:c r="F115" s="107" t="str">
+        <x:v>https://fhir.dghs.gov.bd/core/full-ig.zip</x:v>
+      </x:c>
+      <x:c r="G115" s="107" t="str">
+        <x:v>ZIP documentation package</x:v>
+      </x:c>
+      <x:c r="H115" s="107" t="str">
+        <x:v>Official Bangladesh implementation guide; documents the national Condition and Vaccine terminology bindings used by the project.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="84" customHeight="1">
+      <x:c r="A116" s="107" t="n">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="B116" s="107" t="str">
+        <x:v>Health</x:v>
+      </x:c>
+      <x:c r="C116" s="107" t="str">
+        <x:v>DGHS / MoHFW</x:v>
+      </x:c>
+      <x:c r="D116" s="107" t="str">
+        <x:v>Disease Terminology</x:v>
+      </x:c>
+      <x:c r="E116" s="107" t="str">
+        <x:v>Bangladesh ICD-11 MMS Condition ValueSet (Diagnosis and Finding)</x:v>
+      </x:c>
+      <x:c r="F116" s="107" t="str">
+        <x:v>https://tr.ocl.dghs.gov.bd/api/orgs/MoHFW/collections/bd-condition-icd11-diagnosis-valueset/HEAD/expansions/autoexpand-HEAD/concepts/?limit=1000</x:v>
+      </x:c>
+      <x:c r="G116" s="107" t="str">
+        <x:v>JSON API dataset</x:v>
+      </x:c>
+      <x:c r="H116" s="107" t="str">
+        <x:v>Official national OCL public expansion returned 18,508 unique displayable Condition concepts (13,389 Diagnosis and 5,119 Finding); blank code/name 0.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="84" customHeight="1">
+      <x:c r="A117" s="107" t="n">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="B117" s="107" t="str">
+        <x:v>Health</x:v>
+      </x:c>
+      <x:c r="C117" s="107" t="str">
+        <x:v>DGHS / MoHFW</x:v>
+      </x:c>
+      <x:c r="D117" s="107" t="str">
+        <x:v>Vaccination</x:v>
+      </x:c>
+      <x:c r="E117" s="107" t="str">
+        <x:v>Bangladesh Vaccine Value Set</x:v>
+      </x:c>
+      <x:c r="F117" s="107" t="str">
+        <x:v>https://fhir.dghs.gov.bd/core/ValueSet-bd-vaccine-valueset.html</x:v>
+      </x:c>
+      <x:c r="G117" s="107" t="str">
+        <x:v>HTML/JSON terminology</x:v>
+      </x:c>
+      <x:c r="H117" s="107" t="str">
+        <x:v>Official list of 10 vaccines allowed for immunization in Bangladesh; catalogued as reference evidence, not converted into patient events because PatientID is not published.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="84" customHeight="1">
+      <x:c r="A118" s="107" t="n">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="B118" s="107" t="str">
+        <x:v>Health</x:v>
+      </x:c>
+      <x:c r="C118" s="107" t="str">
+        <x:v>Bangladesh Open Data</x:v>
+      </x:c>
+      <x:c r="D118" s="107" t="str">
+        <x:v>Health Workforce</x:v>
+      </x:c>
+      <x:c r="E118" s="107" t="str">
+        <x:v>Doctor Directory</x:v>
+      </x:c>
+      <x:c r="F118" s="107" t="str">
+        <x:v>https://data.gov.bd/sites/default/files/data-resource/2016/10/18/Doctor-Directory.xls</x:v>
+      </x:c>
+      <x:c r="G118" s="107" t="str">
+        <x:v>XLS dataset</x:v>
+      </x:c>
+      <x:c r="H118" s="107" t="str">
+        <x:v>Official directory has 199 provider rows and 68 raw Post values; 54 clean new Post values map to Designation. HealthWorker rows are withheld because Gender is absent.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f24fe96fec041a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80d6c972f0f84d4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Replace local dataset references with official URLs
</commit_message>
<xml_diff>
--- a/health_data.xlsx
+++ b/health_data.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health" sheetId="8" r:id="Re6c85285bee54932"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health_Catalog_Clean" sheetId="9" r:id="Rb08629cd6dd64ba1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health" sheetId="8" r:id="Re0e1187435774f93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health_Catalog_Clean" sheetId="9" r:id="Rc4fbe0a558024bec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -137,13 +137,7 @@
     <x:t xml:space="preserve">Tuberculosis</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">file:///C:/Users/Hp/Downloads/Annual-Report-2023-unedited-version.pdf</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Dengue</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Revised_National_Guideline_for_Clinical_Management_of_Dengue_Syndrome_2018</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Measels</x:t>
@@ -1885,8 +1879,8 @@
       <x:c r="D17" s="26" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="E17" s="17" t="s">
-        <x:v>42</x:v>
+      <x:c r="E17" s="17" t="str">
+        <x:v>https://www.ntp.gov.bd/wp-content/uploads/2025/04/Annual-Report-2023-unedited-version.pdf</x:v>
       </x:c>
       <x:c r="F17" s="75"/>
       <x:c r="G17" s="46"/>
@@ -1896,10 +1890,10 @@
       <x:c r="B18" s="82"/>
       <x:c r="C18" s="83"/>
       <x:c r="D18" s="49" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="E18" s="16" t="s">
-        <x:v>44</x:v>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E18" s="16" t="str">
+        <x:v>https://old.dghs.gov.bd/images/docs/Publicaations/NationalGuidelineforDengue2018.pdf</x:v>
       </x:c>
       <x:c r="F18" s="75"/>
     </x:row>
@@ -1908,10 +1902,10 @@
       <x:c r="B19" s="82"/>
       <x:c r="C19" s="83"/>
       <x:c r="D19" s="49" t="s">
-        <x:v>45</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E19" s="4" t="s">
-        <x:v>46</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="F19" s="75"/>
       <x:c r="G19" s="46"/>
@@ -1920,13 +1914,13 @@
       <x:c r="A20" s="77"/>
       <x:c r="B20" s="82"/>
       <x:c r="C20" s="7" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="D20" s="27" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="E20" s="4" t="s">
         <x:v>47</x:v>
-      </x:c>
-      <x:c r="D20" s="27" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="E20" s="4" t="s">
-        <x:v>49</x:v>
       </x:c>
       <x:c r="F20" s="75"/>
       <x:c r="G20" s="46"/>
@@ -1935,13 +1929,13 @@
       <x:c r="A21" s="77"/>
       <x:c r="B21" s="82"/>
       <x:c r="C21" s="8" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="D21" s="27" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="E21" s="16" t="s">
         <x:v>50</x:v>
-      </x:c>
-      <x:c r="D21" s="27" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E21" s="16" t="s">
-        <x:v>52</x:v>
       </x:c>
       <x:c r="F21" s="75"/>
     </x:row>
@@ -1949,13 +1943,13 @@
       <x:c r="A22" s="77"/>
       <x:c r="B22" s="82"/>
       <x:c r="C22" s="7" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="D22" s="26" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E22" s="4" t="s">
         <x:v>53</x:v>
-      </x:c>
-      <x:c r="D22" s="26" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E22" s="4" t="s">
-        <x:v>55</x:v>
       </x:c>
       <x:c r="F22" s="75"/>
       <x:c r="G22" s="46"/>
@@ -1964,13 +1958,13 @@
       <x:c r="A23" s="77"/>
       <x:c r="B23" s="82"/>
       <x:c r="C23" s="7" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D23" s="26" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="E23" s="16" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="D23" s="26" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="E23" s="16" t="s">
-        <x:v>58</x:v>
       </x:c>
       <x:c r="F23" s="75"/>
       <x:c r="G23" s="46"/>
@@ -1979,13 +1973,13 @@
       <x:c r="A24" s="77"/>
       <x:c r="B24" s="82"/>
       <x:c r="C24" s="68" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="D24" s="67" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="E24" s="4" t="s">
         <x:v>59</x:v>
-      </x:c>
-      <x:c r="D24" s="67" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="E24" s="4" t="s">
-        <x:v>61</x:v>
       </x:c>
       <x:c r="F24" s="75"/>
       <x:c r="G24" s="46"/>
@@ -1996,7 +1990,7 @@
       <x:c r="C25" s="69"/>
       <x:c r="D25" s="67"/>
       <x:c r="E25" s="16" t="s">
-        <x:v>62</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="F25" s="75"/>
       <x:c r="G25" s="46"/>
@@ -2007,7 +2001,7 @@
       <x:c r="C26" s="69"/>
       <x:c r="D26" s="67"/>
       <x:c r="E26" s="4" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="F26" s="75"/>
       <x:c r="G26" s="46"/>
@@ -2018,7 +2012,7 @@
       <x:c r="C27" s="70"/>
       <x:c r="D27" s="67"/>
       <x:c r="E27" s="16" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="F27" s="75"/>
       <x:c r="G27" s="46"/>
@@ -2026,16 +2020,16 @@
     <x:row r="28" ht="15" customHeight="1">
       <x:c r="A28" s="77"/>
       <x:c r="B28" s="91" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="C28" s="84" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D28" s="49" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="C28" s="84" t="s">
+      <x:c r="E28" s="4" t="s">
         <x:v>66</x:v>
-      </x:c>
-      <x:c r="D28" s="49" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="E28" s="4" t="s">
-        <x:v>68</x:v>
       </x:c>
       <x:c r="F28" s="75"/>
       <x:c r="G28" s="45"/>
@@ -2045,10 +2039,10 @@
       <x:c r="B29" s="91"/>
       <x:c r="C29" s="84"/>
       <x:c r="D29" s="26" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="E29" s="16" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="F29" s="75"/>
       <x:c r="G29" s="45"/>
@@ -2058,10 +2052,10 @@
       <x:c r="B30" s="91"/>
       <x:c r="C30" s="84"/>
       <x:c r="D30" s="49" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E30" s="4" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F30" s="75"/>
       <x:c r="G30" s="45"/>
@@ -2071,10 +2065,10 @@
       <x:c r="B31" s="91"/>
       <x:c r="C31" s="84"/>
       <x:c r="D31" s="49" t="s">
-        <x:v>73</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E31" s="4" t="s">
-        <x:v>74</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="F31" s="75"/>
       <x:c r="G31" s="45"/>
@@ -2084,10 +2078,10 @@
       <x:c r="B32" s="91"/>
       <x:c r="C32" s="84"/>
       <x:c r="D32" s="26" t="s">
-        <x:v>75</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="E32" s="16" t="s">
-        <x:v>76</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="F32" s="75"/>
       <x:c r="G32" s="45"/>
@@ -2097,10 +2091,10 @@
       <x:c r="B33" s="91"/>
       <x:c r="C33" s="84"/>
       <x:c r="D33" s="49" t="s">
-        <x:v>77</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="E33" s="4" t="s">
-        <x:v>78</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F33" s="75"/>
       <x:c r="G33" s="45"/>
@@ -2110,10 +2104,10 @@
       <x:c r="B34" s="91"/>
       <x:c r="C34" s="84"/>
       <x:c r="D34" s="26" t="s">
-        <x:v>79</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E34" s="16" t="s">
-        <x:v>80</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="F34" s="75"/>
       <x:c r="G34" s="45"/>
@@ -2123,10 +2117,10 @@
       <x:c r="B35" s="91"/>
       <x:c r="C35" s="84"/>
       <x:c r="D35" s="49" t="s">
-        <x:v>81</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="E35" s="4" t="s">
-        <x:v>82</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="F35" s="75"/>
       <x:c r="G35" s="45"/>
@@ -2136,10 +2130,10 @@
       <x:c r="B36" s="91"/>
       <x:c r="C36" s="84"/>
       <x:c r="D36" s="26" t="s">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="E36" s="16" t="s">
-        <x:v>84</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="F36" s="75"/>
       <x:c r="G36" s="45"/>
@@ -2149,10 +2143,10 @@
       <x:c r="B37" s="91"/>
       <x:c r="C37" s="84"/>
       <x:c r="D37" s="49" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="E37" s="4" t="s">
-        <x:v>86</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="F37" s="75"/>
       <x:c r="G37" s="45"/>
@@ -2162,10 +2156,10 @@
       <x:c r="B38" s="91"/>
       <x:c r="C38" s="84"/>
       <x:c r="D38" s="26" t="s">
-        <x:v>87</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="E38" s="16" t="s">
-        <x:v>88</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="F38" s="75"/>
       <x:c r="G38" s="45"/>
@@ -2175,10 +2169,10 @@
       <x:c r="B39" s="91"/>
       <x:c r="C39" s="84"/>
       <x:c r="D39" s="49" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E39" s="4" t="s">
-        <x:v>90</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="F39" s="75"/>
       <x:c r="G39" s="45"/>
@@ -2188,10 +2182,10 @@
       <x:c r="B40" s="91"/>
       <x:c r="C40" s="84"/>
       <x:c r="D40" s="26" t="s">
-        <x:v>91</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="E40" s="16" t="s">
-        <x:v>92</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="F40" s="75"/>
       <x:c r="G40" s="45"/>
@@ -2201,10 +2195,10 @@
       <x:c r="B41" s="91"/>
       <x:c r="C41" s="84"/>
       <x:c r="D41" s="26" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="E41" s="16" t="s">
-        <x:v>94</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="F41" s="75"/>
       <x:c r="G41" s="45"/>
@@ -2214,10 +2208,10 @@
       <x:c r="B42" s="91"/>
       <x:c r="C42" s="84"/>
       <x:c r="D42" s="26" t="s">
-        <x:v>95</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="E42" s="16" t="s">
-        <x:v>96</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="F42" s="75"/>
       <x:c r="G42" s="45"/>
@@ -2227,10 +2221,10 @@
       <x:c r="B43" s="91"/>
       <x:c r="C43" s="84"/>
       <x:c r="D43" s="26" t="s">
-        <x:v>97</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="E43" s="16" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="F43" s="75"/>
       <x:c r="G43" s="45"/>
@@ -2240,10 +2234,10 @@
       <x:c r="B44" s="91"/>
       <x:c r="C44" s="84"/>
       <x:c r="D44" s="26" t="s">
-        <x:v>99</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="E44" s="16" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="F44" s="75"/>
       <x:c r="G44" s="45"/>
@@ -2253,10 +2247,10 @@
       <x:c r="B45" s="91"/>
       <x:c r="C45" s="84"/>
       <x:c r="D45" s="26" t="s">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="E45" s="16" t="s">
-        <x:v>102</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="F45" s="75"/>
       <x:c r="G45" s="45"/>
@@ -2265,13 +2259,13 @@
       <x:c r="A46" s="77"/>
       <x:c r="B46" s="91"/>
       <x:c r="C46" s="71" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="D46" s="21" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="E46" s="17" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="D46" s="21" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="E46" s="17" t="s">
-        <x:v>105</x:v>
       </x:c>
       <x:c r="F46" s="75"/>
       <x:c r="G46" s="45"/>
@@ -2282,10 +2276,10 @@
       <x:c r="B47" s="91"/>
       <x:c r="C47" s="72"/>
       <x:c r="D47" s="21" t="s">
-        <x:v>106</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="E47" s="4" t="s">
-        <x:v>107</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="F47" s="75"/>
       <x:c r="G47" s="45"/>
@@ -2296,10 +2290,10 @@
       <x:c r="B48" s="91"/>
       <x:c r="C48" s="72"/>
       <x:c r="D48" s="21" t="s">
-        <x:v>108</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="E48" s="4" t="s">
-        <x:v>109</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="F48" s="75"/>
       <x:c r="G48" s="45"/>
@@ -2310,10 +2304,10 @@
       <x:c r="B49" s="91"/>
       <x:c r="C49" s="72"/>
       <x:c r="D49" s="21" t="s">
-        <x:v>110</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="E49" s="18" t="s">
-        <x:v>111</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="F49" s="75"/>
       <x:c r="G49" s="45"/>
@@ -2324,10 +2318,10 @@
       <x:c r="B50" s="91"/>
       <x:c r="C50" s="72"/>
       <x:c r="D50" s="21" t="s">
-        <x:v>112</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E50" s="17" t="s">
-        <x:v>113</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="F50" s="75"/>
       <x:c r="G50" s="45"/>
@@ -2338,10 +2332,10 @@
       <x:c r="B51" s="91"/>
       <x:c r="C51" s="72"/>
       <x:c r="D51" s="21" t="s">
-        <x:v>114</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="E51" s="17" t="s">
-        <x:v>115</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="F51" s="75"/>
       <x:c r="G51" s="45"/>
@@ -2352,10 +2346,10 @@
       <x:c r="B52" s="91"/>
       <x:c r="C52" s="72"/>
       <x:c r="D52" s="21" t="s">
-        <x:v>116</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="E52" s="17" t="s">
-        <x:v>117</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="F52" s="75"/>
       <x:c r="G52" s="45"/>
@@ -2366,10 +2360,10 @@
       <x:c r="B53" s="91"/>
       <x:c r="C53" s="72"/>
       <x:c r="D53" s="21" t="s">
-        <x:v>118</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="E53" s="17" t="s">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F53" s="75"/>
       <x:c r="G53" s="45"/>
@@ -2380,10 +2374,10 @@
       <x:c r="B54" s="91"/>
       <x:c r="C54" s="72"/>
       <x:c r="D54" s="21" t="s">
-        <x:v>120</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="E54" s="16" t="s">
-        <x:v>121</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F54" s="75"/>
       <x:c r="G54" s="45"/>
@@ -2394,10 +2388,10 @@
       <x:c r="B55" s="91"/>
       <x:c r="C55" s="72"/>
       <x:c r="D55" s="21" t="s">
-        <x:v>122</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="E55" s="4" t="s">
-        <x:v>123</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="F55" s="75"/>
       <x:c r="G55" s="45"/>
@@ -2408,10 +2402,10 @@
       <x:c r="B56" s="91"/>
       <x:c r="C56" s="72"/>
       <x:c r="D56" s="21" t="s">
-        <x:v>124</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E56" s="16" t="s">
-        <x:v>125</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="F56" s="75"/>
       <x:c r="G56" s="45"/>
@@ -2422,10 +2416,10 @@
       <x:c r="B57" s="91"/>
       <x:c r="C57" s="72"/>
       <x:c r="D57" s="21" t="s">
-        <x:v>126</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="E57" s="4" t="s">
-        <x:v>127</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="F57" s="75"/>
       <x:c r="G57" s="45"/>
@@ -2436,10 +2430,10 @@
       <x:c r="B58" s="91"/>
       <x:c r="C58" s="72"/>
       <x:c r="D58" s="21" t="s">
-        <x:v>128</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="E58" s="16" t="s">
-        <x:v>129</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="F58" s="75"/>
       <x:c r="G58" s="45"/>
@@ -2450,10 +2444,10 @@
       <x:c r="B59" s="91"/>
       <x:c r="C59" s="72"/>
       <x:c r="D59" s="21" t="s">
-        <x:v>130</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E59" s="4" t="s">
-        <x:v>131</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="F59" s="75"/>
       <x:c r="G59" s="45"/>
@@ -2464,10 +2458,10 @@
       <x:c r="B60" s="91"/>
       <x:c r="C60" s="72"/>
       <x:c r="D60" s="21" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="E60" s="16" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="F60" s="75"/>
       <x:c r="G60" s="45"/>
@@ -2478,10 +2472,10 @@
       <x:c r="B61" s="91"/>
       <x:c r="C61" s="72"/>
       <x:c r="D61" s="21" t="s">
-        <x:v>134</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="E61" s="4" t="s">
-        <x:v>135</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="F61" s="75"/>
       <x:c r="G61" s="45"/>
@@ -2492,10 +2486,10 @@
       <x:c r="B62" s="91"/>
       <x:c r="C62" s="72"/>
       <x:c r="D62" s="21" t="s">
-        <x:v>136</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="E62" s="16" t="s">
-        <x:v>137</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="F62" s="75"/>
       <x:c r="G62" s="45"/>
@@ -2506,10 +2500,10 @@
       <x:c r="B63" s="91"/>
       <x:c r="C63" s="72"/>
       <x:c r="D63" s="21" t="s">
-        <x:v>138</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="E63" s="16" t="s">
-        <x:v>139</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="F63" s="75"/>
       <x:c r="G63" s="45"/>
@@ -2520,10 +2514,10 @@
       <x:c r="B64" s="91"/>
       <x:c r="C64" s="72"/>
       <x:c r="D64" s="21" t="s">
-        <x:v>140</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="E64" s="16" t="s">
-        <x:v>141</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="F64" s="75"/>
       <x:c r="G64" s="45"/>
@@ -2534,10 +2528,10 @@
       <x:c r="B65" s="91"/>
       <x:c r="C65" s="72"/>
       <x:c r="D65" s="21" t="s">
-        <x:v>142</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="E65" s="16" t="s">
-        <x:v>143</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="F65" s="75"/>
       <x:c r="G65" s="45"/>
@@ -2548,10 +2542,10 @@
       <x:c r="B66" s="91"/>
       <x:c r="C66" s="72"/>
       <x:c r="D66" s="21" t="s">
-        <x:v>144</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="E66" s="16" t="s">
-        <x:v>145</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="F66" s="75"/>
       <x:c r="G66" s="45"/>
@@ -2562,10 +2556,10 @@
       <x:c r="B67" s="91"/>
       <x:c r="C67" s="72"/>
       <x:c r="D67" s="21" t="s">
-        <x:v>146</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="E67" s="16" t="s">
-        <x:v>147</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="F67" s="75"/>
       <x:c r="G67" s="45"/>
@@ -2576,10 +2570,10 @@
       <x:c r="B68" s="91"/>
       <x:c r="C68" s="72"/>
       <x:c r="D68" s="21" t="s">
-        <x:v>148</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="E68" s="16" t="s">
-        <x:v>149</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="F68" s="75"/>
       <x:c r="G68" s="45"/>
@@ -2590,10 +2584,10 @@
       <x:c r="B69" s="91"/>
       <x:c r="C69" s="72"/>
       <x:c r="D69" s="21" t="s">
-        <x:v>150</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="E69" s="16" t="s">
-        <x:v>151</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="F69" s="75"/>
       <x:c r="G69" s="45"/>
@@ -2604,10 +2598,10 @@
       <x:c r="B70" s="91"/>
       <x:c r="C70" s="72"/>
       <x:c r="D70" s="23" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="E70" s="16" t="s">
-        <x:v>153</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="F70" s="75"/>
       <x:c r="G70" s="45"/>
@@ -2618,10 +2612,10 @@
       <x:c r="B71" s="91"/>
       <x:c r="C71" s="72"/>
       <x:c r="D71" s="21" t="s">
-        <x:v>154</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="E71" s="16" t="s">
-        <x:v>155</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="F71" s="75"/>
       <x:c r="G71" s="45"/>
@@ -2632,10 +2626,10 @@
       <x:c r="B72" s="91"/>
       <x:c r="C72" s="72"/>
       <x:c r="D72" s="21" t="s">
-        <x:v>156</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="E72" s="16" t="s">
-        <x:v>157</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="F72" s="75"/>
       <x:c r="G72" s="45"/>
@@ -2646,10 +2640,10 @@
       <x:c r="B73" s="91"/>
       <x:c r="C73" s="73"/>
       <x:c r="D73" s="21" t="s">
-        <x:v>158</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="E73" s="16" t="s">
-        <x:v>159</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="F73" s="75"/>
       <x:c r="G73" s="45"/>
@@ -2659,13 +2653,13 @@
       <x:c r="A74" s="77"/>
       <x:c r="B74" s="91"/>
       <x:c r="C74" s="32" t="s">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D74" s="21" t="s">
-        <x:v>160</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="E74" s="16" t="s">
-        <x:v>161</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="F74" s="75"/>
     </x:row>
@@ -2673,13 +2667,13 @@
       <x:c r="A75" s="77"/>
       <x:c r="B75" s="91"/>
       <x:c r="C75" s="50" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="D75" s="28" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="E75" s="18" t="s">
         <x:v>162</x:v>
-      </x:c>
-      <x:c r="D75" s="28" t="s">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="E75" s="18" t="s">
-        <x:v>164</x:v>
       </x:c>
       <x:c r="F75" s="75"/>
     </x:row>
@@ -2687,13 +2681,13 @@
       <x:c r="A76" s="77"/>
       <x:c r="B76" s="91"/>
       <x:c r="C76" s="84" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="D76" s="29" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="E76" s="18" t="s">
         <x:v>165</x:v>
-      </x:c>
-      <x:c r="D76" s="29" t="s">
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="E76" s="18" t="s">
-        <x:v>167</x:v>
       </x:c>
       <x:c r="F76" s="75"/>
     </x:row>
@@ -2702,10 +2696,10 @@
       <x:c r="B77" s="91"/>
       <x:c r="C77" s="84"/>
       <x:c r="D77" s="29" t="s">
-        <x:v>168</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="E77" s="18" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="F77" s="75"/>
     </x:row>
@@ -2713,13 +2707,13 @@
       <x:c r="A78" s="77"/>
       <x:c r="B78" s="91"/>
       <x:c r="C78" s="50" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="D78" s="26" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="E78" s="18" t="s">
         <x:v>170</x:v>
-      </x:c>
-      <x:c r="D78" s="26" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="E78" s="18" t="s">
-        <x:v>172</x:v>
       </x:c>
       <x:c r="F78" s="75"/>
     </x:row>
@@ -2727,13 +2721,13 @@
       <x:c r="A79" s="77"/>
       <x:c r="B79" s="91"/>
       <x:c r="C79" s="50" t="s">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="D79" s="30" t="s">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="E79" s="18" t="s">
         <x:v>173</x:v>
-      </x:c>
-      <x:c r="D79" s="30" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="E79" s="18" t="s">
-        <x:v>175</x:v>
       </x:c>
       <x:c r="F79" s="75"/>
     </x:row>
@@ -2741,13 +2735,13 @@
       <x:c r="A80" s="77"/>
       <x:c r="B80" s="91"/>
       <x:c r="C80" s="50" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="D80" s="21" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="E80" s="18" t="s">
         <x:v>176</x:v>
-      </x:c>
-      <x:c r="D80" s="21" t="s">
-        <x:v>177</x:v>
-      </x:c>
-      <x:c r="E80" s="18" t="s">
-        <x:v>178</x:v>
       </x:c>
       <x:c r="F80" s="75"/>
     </x:row>
@@ -2755,13 +2749,13 @@
       <x:c r="A81" s="77"/>
       <x:c r="B81" s="91"/>
       <x:c r="C81" s="50" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="D81" s="26" t="s">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="E81" s="18" t="s">
         <x:v>179</x:v>
-      </x:c>
-      <x:c r="D81" s="26" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="E81" s="18" t="s">
-        <x:v>181</x:v>
       </x:c>
       <x:c r="F81" s="75"/>
     </x:row>
@@ -2769,13 +2763,13 @@
       <x:c r="A82" s="77"/>
       <x:c r="B82" s="91"/>
       <x:c r="C82" s="50" t="s">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="D82" s="26" t="s">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="E82" s="18" t="s">
         <x:v>182</x:v>
-      </x:c>
-      <x:c r="D82" s="26" t="s">
-        <x:v>183</x:v>
-      </x:c>
-      <x:c r="E82" s="18" t="s">
-        <x:v>184</x:v>
       </x:c>
       <x:c r="F82" s="75"/>
     </x:row>
@@ -2783,13 +2777,13 @@
       <x:c r="A83" s="77"/>
       <x:c r="B83" s="91"/>
       <x:c r="C83" s="50" t="s">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="D83" s="26" t="s">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="E83" s="18" t="s">
         <x:v>185</x:v>
-      </x:c>
-      <x:c r="D83" s="26" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="E83" s="18" t="s">
-        <x:v>187</x:v>
       </x:c>
       <x:c r="F83" s="75"/>
     </x:row>
@@ -2797,13 +2791,13 @@
       <x:c r="A84" s="77"/>
       <x:c r="B84" s="91"/>
       <x:c r="C84" s="88" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="D84" s="21" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="E84" s="18" t="s">
         <x:v>188</x:v>
-      </x:c>
-      <x:c r="D84" s="21" t="s">
-        <x:v>189</x:v>
-      </x:c>
-      <x:c r="E84" s="18" t="s">
-        <x:v>190</x:v>
       </x:c>
       <x:c r="F84" s="75"/>
     </x:row>
@@ -2812,10 +2806,10 @@
       <x:c r="B85" s="91"/>
       <x:c r="C85" s="89"/>
       <x:c r="D85" s="21" t="s">
-        <x:v>191</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="E85" s="18" t="s">
-        <x:v>192</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="F85" s="75"/>
     </x:row>
@@ -2824,10 +2818,10 @@
       <x:c r="B86" s="91"/>
       <x:c r="C86" s="89"/>
       <x:c r="D86" s="26" t="s">
-        <x:v>193</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="E86" s="18" t="s">
-        <x:v>194</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="F86" s="75"/>
     </x:row>
@@ -2836,10 +2830,10 @@
       <x:c r="B87" s="91"/>
       <x:c r="C87" s="89"/>
       <x:c r="D87" s="26" t="s">
-        <x:v>195</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="E87" s="18" t="s">
-        <x:v>196</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="F87" s="75"/>
     </x:row>
@@ -2848,26 +2842,26 @@
       <x:c r="B88" s="91"/>
       <x:c r="C88" s="90"/>
       <x:c r="D88" s="26" t="s">
-        <x:v>197</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="E88" s="18" t="s">
-        <x:v>198</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="F88" s="75"/>
     </x:row>
     <x:row r="89" ht="28.5" customHeight="1">
       <x:c r="A89" s="77"/>
       <x:c r="B89" s="82" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="C89" s="58" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="D89" s="61" t="s">
         <x:v>199</x:v>
       </x:c>
-      <x:c r="C89" s="58" t="s">
+      <x:c r="E89" s="18" t="s">
         <x:v>200</x:v>
-      </x:c>
-      <x:c r="D89" s="61" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="E89" s="18" t="s">
-        <x:v>202</x:v>
       </x:c>
       <x:c r="F89" s="75"/>
       <x:c r="G89" s="46"/>
@@ -2879,7 +2873,7 @@
       <x:c r="C90" s="59"/>
       <x:c r="D90" s="62"/>
       <x:c r="E90" s="18" t="s">
-        <x:v>203</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="F90" s="75"/>
       <x:c r="G90" s="46"/>
@@ -2891,7 +2885,7 @@
       <x:c r="C91" s="59"/>
       <x:c r="D91" s="62"/>
       <x:c r="E91" s="18" t="s">
-        <x:v>204</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="F91" s="75"/>
       <x:c r="G91" s="46"/>
@@ -2903,7 +2897,7 @@
       <x:c r="C92" s="60"/>
       <x:c r="D92" s="63"/>
       <x:c r="E92" s="18" t="s">
-        <x:v>205</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="F92" s="75"/>
       <x:c r="G92" s="46"/>
@@ -2912,16 +2906,16 @@
     <x:row r="93" ht="15" customHeight="1">
       <x:c r="A93" s="77"/>
       <x:c r="B93" s="80" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="C93" s="78" t="s">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="D93" s="27" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="C93" s="78" t="s">
+      <x:c r="E93" s="18" t="s">
         <x:v>207</x:v>
-      </x:c>
-      <x:c r="D93" s="27" t="s">
-        <x:v>208</x:v>
-      </x:c>
-      <x:c r="E93" s="18" t="s">
-        <x:v>209</x:v>
       </x:c>
       <x:c r="F93" s="75"/>
       <x:c r="G93" s="45"/>
@@ -2932,10 +2926,10 @@
       <x:c r="B94" s="80"/>
       <x:c r="C94" s="79"/>
       <x:c r="D94" s="27" t="s">
-        <x:v>210</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="E94" s="18" t="s">
-        <x:v>211</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="F94" s="75"/>
       <x:c r="G94" s="45"/>
@@ -2946,10 +2940,10 @@
       <x:c r="B95" s="80"/>
       <x:c r="C95" s="79"/>
       <x:c r="D95" s="27" t="s">
-        <x:v>212</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="E95" s="18" t="s">
-        <x:v>213</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="F95" s="75"/>
       <x:c r="G95" s="45"/>
@@ -2960,10 +2954,10 @@
       <x:c r="B96" s="80"/>
       <x:c r="C96" s="79"/>
       <x:c r="D96" s="27" t="s">
-        <x:v>214</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="E96" s="18" t="s">
-        <x:v>215</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="F96" s="75"/>
       <x:c r="G96" s="45"/>
@@ -2974,10 +2968,10 @@
       <x:c r="B97" s="80"/>
       <x:c r="C97" s="79"/>
       <x:c r="D97" s="31" t="s">
-        <x:v>216</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="E97" s="18" t="s">
-        <x:v>217</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="F97" s="75"/>
       <x:c r="G97" s="45"/>
@@ -2988,10 +2982,10 @@
       <x:c r="B98" s="80"/>
       <x:c r="C98" s="79"/>
       <x:c r="D98" s="27" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="E98" s="18" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="F98" s="75"/>
       <x:c r="G98" s="45"/>
@@ -3002,10 +2996,10 @@
       <x:c r="B99" s="80"/>
       <x:c r="C99" s="79"/>
       <x:c r="D99" s="27" t="s">
-        <x:v>220</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="E99" s="18" t="s">
-        <x:v>221</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="F99" s="75"/>
       <x:c r="G99" s="45"/>
@@ -3016,10 +3010,10 @@
       <x:c r="B100" s="80"/>
       <x:c r="C100" s="79"/>
       <x:c r="D100" s="27" t="s">
-        <x:v>222</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="E100" s="18" t="s">
-        <x:v>223</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="F100" s="75"/>
       <x:c r="G100" s="45"/>
@@ -3030,10 +3024,10 @@
       <x:c r="B101" s="80"/>
       <x:c r="C101" s="79"/>
       <x:c r="D101" s="27" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="E101" s="18" t="s">
-        <x:v>225</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="F101" s="75"/>
       <x:c r="G101" s="45"/>
@@ -3042,16 +3036,16 @@
     <x:row r="102" ht="15.75" customHeight="1">
       <x:c r="A102" s="77"/>
       <x:c r="B102" s="86" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="C102" s="51" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="D102" s="33" t="s">
         <x:v>226</x:v>
       </x:c>
-      <x:c r="C102" s="51" t="s">
+      <x:c r="E102" s="19" t="s">
         <x:v>227</x:v>
-      </x:c>
-      <x:c r="D102" s="33" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="E102" s="19" t="s">
-        <x:v>229</x:v>
       </x:c>
       <x:c r="F102" s="75"/>
       <x:c r="G102" s="46"/>
@@ -3060,13 +3054,13 @@
       <x:c r="A103" s="77"/>
       <x:c r="B103" s="87"/>
       <x:c r="C103" s="51" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="D103" s="33" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="E103" s="18" t="s">
         <x:v>230</x:v>
-      </x:c>
-      <x:c r="D103" s="33" t="s">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="E103" s="18" t="s">
-        <x:v>232</x:v>
       </x:c>
       <x:c r="F103" s="75"/>
       <x:c r="G103" s="46"/>
@@ -3074,16 +3068,16 @@
     <x:row r="104" ht="15" customHeight="1">
       <x:c r="A104" s="77"/>
       <x:c r="B104" s="57" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="C104" s="55" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="D104" s="33" t="s">
         <x:v>233</x:v>
       </x:c>
-      <x:c r="C104" s="55" t="s">
+      <x:c r="E104" s="37" t="s">
         <x:v>234</x:v>
-      </x:c>
-      <x:c r="D104" s="33" t="s">
-        <x:v>235</x:v>
-      </x:c>
-      <x:c r="E104" s="37" t="s">
-        <x:v>236</x:v>
       </x:c>
       <x:c r="F104" s="75"/>
     </x:row>
@@ -3092,10 +3086,10 @@
       <x:c r="B105" s="57"/>
       <x:c r="C105" s="56"/>
       <x:c r="D105" s="33" t="s">
-        <x:v>237</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="E105" s="37" t="s">
-        <x:v>238</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="F105" s="75"/>
       <x:c r="H105" s="41"/>
@@ -3149,10 +3143,10 @@
       <x:c r="B106" s="57"/>
       <x:c r="C106" s="56"/>
       <x:c r="D106" s="33" t="s">
-        <x:v>239</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="E106" s="37" t="s">
-        <x:v>240</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="F106" s="75"/>
       <x:c r="H106" s="41"/>
@@ -3206,10 +3200,10 @@
       <x:c r="B107" s="57"/>
       <x:c r="C107" s="56"/>
       <x:c r="D107" s="33" t="s">
-        <x:v>241</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="E107" s="37" t="s">
-        <x:v>242</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="F107" s="75"/>
       <x:c r="H107" s="41"/>
@@ -3263,10 +3257,10 @@
       <x:c r="B108" s="57"/>
       <x:c r="C108" s="56"/>
       <x:c r="D108" s="33" t="s">
-        <x:v>243</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="E108" s="37" t="s">
-        <x:v>244</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="F108" s="75"/>
       <x:c r="H108" s="41"/>
@@ -3320,10 +3314,10 @@
       <x:c r="B109" s="57"/>
       <x:c r="C109" s="56"/>
       <x:c r="D109" s="33" t="s">
-        <x:v>245</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="E109" s="37" t="s">
-        <x:v>246</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="F109" s="75"/>
       <x:c r="H109" s="41"/>
@@ -3377,10 +3371,10 @@
       <x:c r="B110" s="57"/>
       <x:c r="C110" s="56"/>
       <x:c r="D110" s="33" t="s">
-        <x:v>247</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="E110" s="37" t="s">
-        <x:v>248</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="F110" s="75"/>
       <x:c r="H110" s="41"/>
@@ -3434,10 +3428,10 @@
       <x:c r="B111" s="57"/>
       <x:c r="C111" s="56"/>
       <x:c r="D111" s="33" t="s">
-        <x:v>249</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="E111" s="37" t="s">
-        <x:v>250</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="F111" s="75"/>
       <x:c r="H111" s="41"/>
@@ -3491,10 +3485,10 @@
       <x:c r="B112" s="57"/>
       <x:c r="C112" s="56"/>
       <x:c r="D112" s="34" t="s">
-        <x:v>251</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="E112" s="37" t="s">
-        <x:v>252</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="F112" s="75"/>
       <x:c r="H112" s="41"/>
@@ -3548,10 +3542,10 @@
       <x:c r="B113" s="57"/>
       <x:c r="C113" s="56"/>
       <x:c r="D113" s="35" t="s">
-        <x:v>253</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="E113" s="38" t="s">
-        <x:v>254</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="F113" s="76"/>
       <x:c r="H113" s="41"/>
@@ -3953,121 +3947,121 @@
     <x:mergeCell ref="C46:C73"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="R36ddba68a1f04fe1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="R4e7a14adfdb14668"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="R90ab7d3a8cf04880"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="R79995dcaa27e4a7c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="R793ef01277f8472a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="R6505d1c87e6b42a4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="R665346b961c84809"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="R45c394ee2cc242fd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="Rb3cc8326818646d9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="Re94a9515ae274edc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="Re1dbf4db9a604481"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="R813df0a08cc1431c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="R4b5f9cb847e94210"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="Rdecdb73b19284c69"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="Rd56d296a350d4d3d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="Ra50138f25f6241d9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="R7f98fbc72f3a4a29"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="Rf3eb8187664c4fd3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="R8749f284a79242c1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="Rce7244587f9b4bd7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="R3e8a65b64e6c42c8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="Rd489d7ab263e47e6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="Ra2f9b2b84e124453"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="R4d5989604c97481b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="Rc86ae9da22fa4f12"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="R749dbbe8a302465e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="R5570de8f0c9b4966"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="R7bdbcb9c364443ae"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="R4710309807a94b66"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="R49590d20cc7c4a36"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="R12ed0e47d2624fe4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="R8c49a1d9f4644f07"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R7de31df136a143b6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="R71944336d7774d46"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="R859c4636b1e748dc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="R06ff2ed70d54485a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="Re074c1ab40584bcb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="Rabf54c231cc54815"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R8958b702c8044c31"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rc980cabc6f394253"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="Rd3f4207fbe094f84"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="R6294ef5eb7a0406f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Rbd43c50f79b54204"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="R1785cf1ef51c4d63"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="Rd2642835bd594f99"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="R283f7fb16baa4a1d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="Rdf2eedd3892b4311"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="R849809ff01514dde"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="Rcf6cca5986314771"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="Race942c77f254553"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R0b8a8283bf2546c0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R1fd0cba662f04a2b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="Rd03b368863b944ba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="R1df572a66233492c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="R846ac1d639d2438e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="Raae4ced769074d5a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R82af723d29874815"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="Rd0dcc5722e8d480e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="Ra44203f3f5164aa7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="Rd531f6d9a57e432b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="Rc0fca617cfde4bbe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R5207eb9f364247c0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R646247e510ba4f70"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="Rfc4550a2437f490d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="Rc8ff2aa94f644a68"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R95ebe06dcfa04742"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="Rc49bba91a80b44e1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="Rf7a254356a76403c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="R440d256b219b471e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="Rba123870283e4002"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="R7af6d91f4fd94e87"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="R418738121aee4f30"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="Rc405e02e810c4a8b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="R48a151732c014d41"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="Rb97f864d4c3b48de"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="R324b64de71b842a6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="R60860006ab95451b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="Rc23473f7d13648f5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="R29147ab062c6474c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="R17f0684390164683"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="R99377a2c4d444008"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="R62a75d42c59b4465"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="Rd19dd137b8264a1c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="Rc58bf10ae50f4871"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="Rfa7eb017486248a8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="R960de8a0500a420f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="Reb66f06851d042a0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="Rc8d113c17e9140ae"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="R0b2f8914f328405a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="Rdf16254457e54898"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="Rf67cea24d2f841f4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="R473e419ac01440fe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="Rfa876d1701644633"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="R3f65a3b016764a3a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="R005fb229c9c64059"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="Re030a500411c419d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="R8a2fe413b83042cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="R1fb8cd498b34499a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="Rb0b88fc334084ee2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="R74f4e4bfc10b4ba8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="R7c58925147644329"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="R94d740552e094563"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="R5c46acfa95144c4f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="R9d7c6aa6a5b140cb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="R7381b6698c9441f8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="R46b57811d2b64e69"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="Rd53defb9c6d54e58"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="R62ad20ccbec748b9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="Ra288e2f6d4274a0e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="Re848affd58954c3d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="Rfe5a752fa5244c38"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="R8a205ef2daff499f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="R1bd3e490e6cf42ad"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="R38d96ff035db472e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="R3be718fc31cf4aae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="R134caf29bb3d4377"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="R3eec689893804f00"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="R3f61182304fe4768"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="Ra38a681c49534379"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="R2b1a74d6bc464e7d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="R8b3d870a8e174306"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="R4509be953eab4586"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="R5f35b21d3b304887"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="Rf2f5345afa2b46c3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="Re208369d06394e2e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="R55768a70f40944fa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="R59d90803c76c4178"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="R9eaa3cb8ebe64be7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="Raa8af87e911847c3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="Rddfaece3c0d04f7f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="R7859c404d4a74ed2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="Rd4288d7c334542a3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="R6fa69b0cc2a8484e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="R80de0637f58e427e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="R523d343e14524e13"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="R18b4059af93049a2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="R7cff4c608fb34d19"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="R1ae24a86e83a41f8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="Rcf9709d8072b4089"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="R21e19fb343754a28"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="Rae3c57129da14355"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="Rf3fb70f07c4245d6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="R44525a9679954621"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="Rc5e533245a794131"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="Rf75c5f1caa574c7c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="R2b5b0604248847cc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="R53d7d46ecc7e43e0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R10926df0ba7d4c27"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="R8f10dee7d2c14287"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="R27c2423b4f1541bc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="R028a44e38e584812"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="Rb0e691f4cc3b41ea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="R8f23742de8004e93"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R8f496140c0444c13"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R00fcbda17a3b4ed4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="R8383b4704f254f25"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="Rfa2110b449d44fdc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Raa5310d1db6747c3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="Rf9e8da0c4f754ba2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="R6e38084bd33a4915"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="R2feb18646ea74c07"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="R0dc0ff68aa124fe0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="R5d3c6af831a54f67"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="R9b563b8d65674de0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="Rf59301754dab48d0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R7d21f391c8444ed3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="Red8968d938b64cb3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="R3fc59f5623fd4600"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="R4b27fd9dbbae47a2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="Rc95dc2f865ca438e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="Rfaa8c17410e74c12"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R3976f9adf6e34348"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="R80e8cf2462bf4fae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="R14f41827dc65425d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="R8cfca85de9fe49d9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="R9f120992403541d1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R9a0a25df79414695"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R05b27db3ae2a424e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="R44b8800581d84701"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="Rc63d776d2bf145dc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R0d3f0e5197694bb0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="Rd158a0890ea2412f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="R93437fe83fbf4453"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="Ra8c1afdcc3754a83"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="Ra9badb1d0a4f4fb6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="Rae63746aea324c9f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="R856df7cb9ab04b67"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="R424e5b94209c4a68"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="Ra1b0405776384e59"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="R3d1ca8aeade2427c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="R5783ed290c0a47bd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="Rbb0f0f373a7b4588"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="R5231c36c0fd34ff4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="Ra5d12da25aa54937"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="Rfb71254d29744d1e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="Rcd09bb75652341a3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="Rbc2d982eba5c428e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="Ra0a1ca5f3606458c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="R4d364f72d4354156"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="R392ecf656e334710"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="R4472aa94850a4076"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="Raae7b97b746149e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="R5912c868210e46d1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="R9e9e82bfee4247cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="R570b635fbf4e40d5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="Raba6a021ca534b56"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="R48aa918e3d684bec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="R53e761b19d1b44e8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="Re9840a83804f43dd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="Ra29ebc5c309d4366"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="R185b288c5e8a4021"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="R50e1af5254934e64"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="Rac26eae02c3b4c94"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="Rb5b808896b664715"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="R011a2ca01aae41a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="R10817c597f7f4c97"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="R95a87f32e37c44e4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="Rc1be0388a4194bc3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="R4fac923dc54c4e6c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="Rd96ae88cb3304743"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="Rb72fe2469a664aa8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="R9a9c922a6c2f4b40"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="R2e787d516c0e43e5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="R125691a2c42b4e04"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="Rcef58b2af86c463b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="Rba97bc8c0e6747cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="R7d234d0b6b2b4fa8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="Rf6bbc43a6b8349f9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="R515564bb153a4f68"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="Rbf23fbb517fb44c3"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4520,7 +4514,7 @@
         <x:v>Tuberculosis</x:v>
       </x:c>
       <x:c r="F17" s="110" t="str">
-        <x:v>file:///C:/Users/Hp/Downloads/Annual-Report-2023-unedited-version.pdf</x:v>
+        <x:v>https://www.ntp.gov.bd/wp-content/uploads/2025/04/Annual-Report-2023-unedited-version.pdf</x:v>
       </x:c>
       <x:c r="G17" s="108" t="str">
         <x:v>PDF document</x:v>
@@ -4546,7 +4540,7 @@
         <x:v>Dengue</x:v>
       </x:c>
       <x:c r="F18" s="110" t="str">
-        <x:v>Revised_National_Guideline_for_Clinical_Management_of_Dengue_Syndrome_2018</x:v>
+        <x:v>https://old.dghs.gov.bd/images/docs/Publicaations/NationalGuidelineforDengue2018.pdf</x:v>
       </x:c>
       <x:c r="G18" s="108" t="str">
         <x:v>PDF document</x:v>
@@ -7158,7 +7152,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80d6c972f0f84d4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54f1c8c698ef491b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify reviewer navigation and source archive naming
</commit_message>
<xml_diff>
--- a/health_data.xlsx
+++ b/health_data.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health" sheetId="8" r:id="Re0e1187435774f93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health_Catalog_Clean" sheetId="9" r:id="Rc4fbe0a558024bec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health" sheetId="8" r:id="Reef434e3809e4215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Health_Catalog_Clean" sheetId="9" r:id="Rd920a9a8bf0941e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,9 +140,6 @@
     <x:t xml:space="preserve">Dengue</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Measels</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.who.int/emergencies/disease-outbreak-news/item/2026-DON598</x:t>
   </x:si>
   <x:si>
@@ -176,18 +173,12 @@
     <x:t xml:space="preserve">Mental Health</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Preventation and Management of Mental Health Conditions in Bangladesh</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://cdn.who.int/media/docs/default-source/mental-health/special-initiative/mhic-bangladesh-report-25.07.25v2.pdf?sfvrsn=7f87a3c6_3</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Maternal Health</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">United Nations Populations fund</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.unfpa.org/sites/default/files/portal-document/ENG_DP.FPA_.CPD_.BGD_.10%20-%20Bangladesh%20CPD%20-%20FINAL%20-%2018Jul21.pdf</x:t>
   </x:si>
   <x:si>
@@ -515,12 +506,6 @@
     <x:t xml:space="preserve">https://old.dghs.gov.bd/images/docs/Publicaations/Cancer%20registry_2.pdf</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Maternal Morality</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bangladesh Maternal Morality Servey</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://old.dghs.gov.bd/licts_file/images/BMMS/BMMS_2010_color.pdf</x:t>
   </x:si>
   <x:si>
@@ -533,45 +518,27 @@
     <x:t xml:space="preserve">https://dghs.gov.bd/pages/notices/mapping-of-the-infectious-disease-surveillance-system-in-bangladesh-ui6g5n-698975c215676b17b1e61d41</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve"> Research Abstract</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Research Abstract of Planning, Monitoring and Research Operational Plan 2021-2022</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://old.dghs.gov.bd/images/docs/Guideline/research_abstract_2021_2022.pdf</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Rohinga Heath Bulletin</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> Rohinga Health Bulletin 2018</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://old.dghs.gov.bd/images/docs/Publicaations/HB_030718.pdf</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">E-Health</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">eHealth Auguest 2012</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://old.dghs.gov.bd/licts_file/images/eHealth/our_eHealth_Aug_2012.pdf</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Climate</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">বাংলাদেশের স্বাস্থ্য খাতে জল-বায়ু পরিবর্তনের প্রভাব (২০০৯ সালে কোপেনহেগেন কপ ১৫ উপলক্ষে প্রস্তুতকৃত)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://old.dghs.gov.bd/licts_file/images/Climate_Change/2009_ClimateChange2009.pdf</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Measles and Rebella Bulletin</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">MR bulletin ( 2nd quarter 2021)</x:t>
   </x:si>
   <x:si>
@@ -605,12 +572,6 @@
     <x:t xml:space="preserve">NICVD</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">National Institute of cardiovascular Disease</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cardiovascular Diseases  Information</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://pub.flowpaper.com/docs/https:/www.nicvd.gov.bd/uploadFile/journal/40dbe_5098.pdf</x:t>
   </x:si>
   <x:si>
@@ -627,9 +588,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Policy and Administration</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">বাংলাদেশ হেলথ ওয়ার্কফোর্স স্ট্রাটেজি ২০২৪</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://objectstorage.ap-dcc-gazipur-1.oraclecloud15.com/n/axvjbnqprylg/b/V2Ministry/o/office-hsd/2024/12/ab1c3ee0b4a54a69a4e3044865b01e23.pdf</x:t>
@@ -1901,11 +1859,11 @@
       <x:c r="A19" s="77"/>
       <x:c r="B19" s="82"/>
       <x:c r="C19" s="83"/>
-      <x:c r="D19" s="49" t="s">
+      <x:c r="D19" s="49" t="str">
+        <x:v>Measles</x:v>
+      </x:c>
+      <x:c r="E19" s="4" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="E19" s="4" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="F19" s="75"/>
       <x:c r="G19" s="46"/>
@@ -1914,13 +1872,13 @@
       <x:c r="A20" s="77"/>
       <x:c r="B20" s="82"/>
       <x:c r="C20" s="7" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D20" s="27" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="D20" s="27" t="s">
+      <x:c r="E20" s="4" t="s">
         <x:v>46</x:v>
-      </x:c>
-      <x:c r="E20" s="4" t="s">
-        <x:v>47</x:v>
       </x:c>
       <x:c r="F20" s="75"/>
       <x:c r="G20" s="46"/>
@@ -1929,13 +1887,13 @@
       <x:c r="A21" s="77"/>
       <x:c r="B21" s="82"/>
       <x:c r="C21" s="8" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="D21" s="27" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="D21" s="27" t="s">
+      <x:c r="E21" s="16" t="s">
         <x:v>49</x:v>
-      </x:c>
-      <x:c r="E21" s="16" t="s">
-        <x:v>50</x:v>
       </x:c>
       <x:c r="F21" s="75"/>
     </x:row>
@@ -1943,13 +1901,13 @@
       <x:c r="A22" s="77"/>
       <x:c r="B22" s="82"/>
       <x:c r="C22" s="7" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D22" s="26" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="D22" s="26" t="s">
+      <x:c r="E22" s="4" t="s">
         <x:v>52</x:v>
-      </x:c>
-      <x:c r="E22" s="4" t="s">
-        <x:v>53</x:v>
       </x:c>
       <x:c r="F22" s="75"/>
       <x:c r="G22" s="46"/>
@@ -1958,13 +1916,13 @@
       <x:c r="A23" s="77"/>
       <x:c r="B23" s="82"/>
       <x:c r="C23" s="7" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="D23" s="26" t="str">
+        <x:v>Prevention and Management of Mental Health Conditions in Bangladesh</x:v>
+      </x:c>
+      <x:c r="E23" s="16" t="s">
         <x:v>54</x:v>
-      </x:c>
-      <x:c r="D23" s="26" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="E23" s="16" t="s">
-        <x:v>56</x:v>
       </x:c>
       <x:c r="F23" s="75"/>
       <x:c r="G23" s="46"/>
@@ -1973,13 +1931,13 @@
       <x:c r="A24" s="77"/>
       <x:c r="B24" s="82"/>
       <x:c r="C24" s="68" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="D24" s="67" t="s">
-        <x:v>58</x:v>
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D24" s="67" t="str">
+        <x:v>UNFPA Country Programme Document for Bangladesh 2022-2026</x:v>
       </x:c>
       <x:c r="E24" s="4" t="s">
-        <x:v>59</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="F24" s="75"/>
       <x:c r="G24" s="46"/>
@@ -1988,9 +1946,11 @@
       <x:c r="A25" s="77"/>
       <x:c r="B25" s="82"/>
       <x:c r="C25" s="69"/>
-      <x:c r="D25" s="67"/>
+      <x:c r="D25" s="67" t="str">
+        <x:v>UNFPA Country Programme Document for Bangladesh 2017-2020</x:v>
+      </x:c>
       <x:c r="E25" s="16" t="s">
-        <x:v>60</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F25" s="75"/>
       <x:c r="G25" s="46"/>
@@ -1999,9 +1959,11 @@
       <x:c r="A26" s="77"/>
       <x:c r="B26" s="82"/>
       <x:c r="C26" s="69"/>
-      <x:c r="D26" s="67"/>
+      <x:c r="D26" s="67" t="str">
+        <x:v>UNDAF Action Plan Bangladesh 2012-2016</x:v>
+      </x:c>
       <x:c r="E26" s="4" t="s">
-        <x:v>61</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="F26" s="75"/>
       <x:c r="G26" s="46"/>
@@ -2010,9 +1972,11 @@
       <x:c r="A27" s="77"/>
       <x:c r="B27" s="82"/>
       <x:c r="C27" s="70"/>
-      <x:c r="D27" s="67"/>
+      <x:c r="D27" s="67" t="str">
+        <x:v>UNFPA Final Country Programme Document for Bangladesh 2012-2016</x:v>
+      </x:c>
       <x:c r="E27" s="16" t="s">
-        <x:v>62</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="F27" s="75"/>
       <x:c r="G27" s="46"/>
@@ -2020,16 +1984,16 @@
     <x:row r="28" ht="15" customHeight="1">
       <x:c r="A28" s="77"/>
       <x:c r="B28" s="91" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C28" s="84" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="D28" s="49" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="E28" s="4" t="s">
         <x:v>63</x:v>
-      </x:c>
-      <x:c r="C28" s="84" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="D28" s="49" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="E28" s="4" t="s">
-        <x:v>66</x:v>
       </x:c>
       <x:c r="F28" s="75"/>
       <x:c r="G28" s="45"/>
@@ -2039,10 +2003,10 @@
       <x:c r="B29" s="91"/>
       <x:c r="C29" s="84"/>
       <x:c r="D29" s="26" t="s">
-        <x:v>67</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E29" s="16" t="s">
-        <x:v>68</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F29" s="75"/>
       <x:c r="G29" s="45"/>
@@ -2052,10 +2016,10 @@
       <x:c r="B30" s="91"/>
       <x:c r="C30" s="84"/>
       <x:c r="D30" s="49" t="s">
-        <x:v>69</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E30" s="4" t="s">
-        <x:v>70</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="F30" s="75"/>
       <x:c r="G30" s="45"/>
@@ -2065,10 +2029,10 @@
       <x:c r="B31" s="91"/>
       <x:c r="C31" s="84"/>
       <x:c r="D31" s="49" t="s">
-        <x:v>71</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E31" s="4" t="s">
-        <x:v>72</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F31" s="75"/>
       <x:c r="G31" s="45"/>
@@ -2078,10 +2042,10 @@
       <x:c r="B32" s="91"/>
       <x:c r="C32" s="84"/>
       <x:c r="D32" s="26" t="s">
-        <x:v>73</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E32" s="16" t="s">
-        <x:v>74</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F32" s="75"/>
       <x:c r="G32" s="45"/>
@@ -2091,10 +2055,10 @@
       <x:c r="B33" s="91"/>
       <x:c r="C33" s="84"/>
       <x:c r="D33" s="49" t="s">
-        <x:v>75</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E33" s="4" t="s">
-        <x:v>76</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="F33" s="75"/>
       <x:c r="G33" s="45"/>
@@ -2104,10 +2068,10 @@
       <x:c r="B34" s="91"/>
       <x:c r="C34" s="84"/>
       <x:c r="D34" s="26" t="s">
-        <x:v>77</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="E34" s="16" t="s">
-        <x:v>78</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="F34" s="75"/>
       <x:c r="G34" s="45"/>
@@ -2117,10 +2081,10 @@
       <x:c r="B35" s="91"/>
       <x:c r="C35" s="84"/>
       <x:c r="D35" s="49" t="s">
-        <x:v>79</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E35" s="4" t="s">
-        <x:v>80</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F35" s="75"/>
       <x:c r="G35" s="45"/>
@@ -2130,10 +2094,10 @@
       <x:c r="B36" s="91"/>
       <x:c r="C36" s="84"/>
       <x:c r="D36" s="26" t="s">
-        <x:v>81</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E36" s="16" t="s">
-        <x:v>82</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="F36" s="75"/>
       <x:c r="G36" s="45"/>
@@ -2143,10 +2107,10 @@
       <x:c r="B37" s="91"/>
       <x:c r="C37" s="84"/>
       <x:c r="D37" s="49" t="s">
-        <x:v>83</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E37" s="4" t="s">
-        <x:v>84</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="F37" s="75"/>
       <x:c r="G37" s="45"/>
@@ -2156,10 +2120,10 @@
       <x:c r="B38" s="91"/>
       <x:c r="C38" s="84"/>
       <x:c r="D38" s="26" t="s">
-        <x:v>85</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="E38" s="16" t="s">
-        <x:v>86</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="F38" s="75"/>
       <x:c r="G38" s="45"/>
@@ -2169,10 +2133,10 @@
       <x:c r="B39" s="91"/>
       <x:c r="C39" s="84"/>
       <x:c r="D39" s="49" t="s">
-        <x:v>87</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E39" s="4" t="s">
-        <x:v>88</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="F39" s="75"/>
       <x:c r="G39" s="45"/>
@@ -2182,10 +2146,10 @@
       <x:c r="B40" s="91"/>
       <x:c r="C40" s="84"/>
       <x:c r="D40" s="26" t="s">
-        <x:v>89</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="E40" s="16" t="s">
-        <x:v>90</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="F40" s="75"/>
       <x:c r="G40" s="45"/>
@@ -2195,10 +2159,10 @@
       <x:c r="B41" s="91"/>
       <x:c r="C41" s="84"/>
       <x:c r="D41" s="26" t="s">
-        <x:v>91</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="E41" s="16" t="s">
-        <x:v>92</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="F41" s="75"/>
       <x:c r="G41" s="45"/>
@@ -2208,10 +2172,10 @@
       <x:c r="B42" s="91"/>
       <x:c r="C42" s="84"/>
       <x:c r="D42" s="26" t="s">
-        <x:v>93</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E42" s="16" t="s">
-        <x:v>94</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="F42" s="75"/>
       <x:c r="G42" s="45"/>
@@ -2221,10 +2185,10 @@
       <x:c r="B43" s="91"/>
       <x:c r="C43" s="84"/>
       <x:c r="D43" s="26" t="s">
-        <x:v>95</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E43" s="16" t="s">
-        <x:v>96</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="F43" s="75"/>
       <x:c r="G43" s="45"/>
@@ -2234,10 +2198,10 @@
       <x:c r="B44" s="91"/>
       <x:c r="C44" s="84"/>
       <x:c r="D44" s="26" t="s">
-        <x:v>97</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="E44" s="16" t="s">
-        <x:v>98</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="F44" s="75"/>
       <x:c r="G44" s="45"/>
@@ -2247,10 +2211,10 @@
       <x:c r="B45" s="91"/>
       <x:c r="C45" s="84"/>
       <x:c r="D45" s="26" t="s">
-        <x:v>99</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E45" s="16" t="s">
-        <x:v>100</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="F45" s="75"/>
       <x:c r="G45" s="45"/>
@@ -2259,13 +2223,13 @@
       <x:c r="A46" s="77"/>
       <x:c r="B46" s="91"/>
       <x:c r="C46" s="71" t="s">
-        <x:v>101</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D46" s="21" t="s">
-        <x:v>102</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="E46" s="17" t="s">
-        <x:v>103</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="F46" s="75"/>
       <x:c r="G46" s="45"/>
@@ -2276,10 +2240,10 @@
       <x:c r="B47" s="91"/>
       <x:c r="C47" s="72"/>
       <x:c r="D47" s="21" t="s">
-        <x:v>104</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="E47" s="4" t="s">
-        <x:v>105</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="F47" s="75"/>
       <x:c r="G47" s="45"/>
@@ -2290,10 +2254,10 @@
       <x:c r="B48" s="91"/>
       <x:c r="C48" s="72"/>
       <x:c r="D48" s="21" t="s">
-        <x:v>106</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="E48" s="4" t="s">
-        <x:v>107</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="F48" s="75"/>
       <x:c r="G48" s="45"/>
@@ -2304,10 +2268,10 @@
       <x:c r="B49" s="91"/>
       <x:c r="C49" s="72"/>
       <x:c r="D49" s="21" t="s">
-        <x:v>108</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="E49" s="18" t="s">
-        <x:v>109</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="F49" s="75"/>
       <x:c r="G49" s="45"/>
@@ -2318,10 +2282,10 @@
       <x:c r="B50" s="91"/>
       <x:c r="C50" s="72"/>
       <x:c r="D50" s="21" t="s">
-        <x:v>110</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E50" s="17" t="s">
-        <x:v>111</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F50" s="75"/>
       <x:c r="G50" s="45"/>
@@ -2332,10 +2296,10 @@
       <x:c r="B51" s="91"/>
       <x:c r="C51" s="72"/>
       <x:c r="D51" s="21" t="s">
-        <x:v>112</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="E51" s="17" t="s">
-        <x:v>113</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="F51" s="75"/>
       <x:c r="G51" s="45"/>
@@ -2346,10 +2310,10 @@
       <x:c r="B52" s="91"/>
       <x:c r="C52" s="72"/>
       <x:c r="D52" s="21" t="s">
-        <x:v>114</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="E52" s="17" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="F52" s="75"/>
       <x:c r="G52" s="45"/>
@@ -2360,10 +2324,10 @@
       <x:c r="B53" s="91"/>
       <x:c r="C53" s="72"/>
       <x:c r="D53" s="21" t="s">
-        <x:v>116</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E53" s="17" t="s">
-        <x:v>117</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="F53" s="75"/>
       <x:c r="G53" s="45"/>
@@ -2374,10 +2338,10 @@
       <x:c r="B54" s="91"/>
       <x:c r="C54" s="72"/>
       <x:c r="D54" s="21" t="s">
-        <x:v>118</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="E54" s="16" t="s">
-        <x:v>119</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="F54" s="75"/>
       <x:c r="G54" s="45"/>
@@ -2388,10 +2352,10 @@
       <x:c r="B55" s="91"/>
       <x:c r="C55" s="72"/>
       <x:c r="D55" s="21" t="s">
-        <x:v>120</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E55" s="4" t="s">
-        <x:v>121</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="F55" s="75"/>
       <x:c r="G55" s="45"/>
@@ -2402,10 +2366,10 @@
       <x:c r="B56" s="91"/>
       <x:c r="C56" s="72"/>
       <x:c r="D56" s="21" t="s">
-        <x:v>122</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="E56" s="16" t="s">
-        <x:v>123</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="F56" s="75"/>
       <x:c r="G56" s="45"/>
@@ -2416,10 +2380,10 @@
       <x:c r="B57" s="91"/>
       <x:c r="C57" s="72"/>
       <x:c r="D57" s="21" t="s">
-        <x:v>124</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="E57" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F57" s="75"/>
       <x:c r="G57" s="45"/>
@@ -2430,10 +2394,10 @@
       <x:c r="B58" s="91"/>
       <x:c r="C58" s="72"/>
       <x:c r="D58" s="21" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="E58" s="16" t="s">
-        <x:v>127</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="F58" s="75"/>
       <x:c r="G58" s="45"/>
@@ -2444,10 +2408,10 @@
       <x:c r="B59" s="91"/>
       <x:c r="C59" s="72"/>
       <x:c r="D59" s="21" t="s">
-        <x:v>128</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="E59" s="4" t="s">
-        <x:v>129</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F59" s="75"/>
       <x:c r="G59" s="45"/>
@@ -2458,10 +2422,10 @@
       <x:c r="B60" s="91"/>
       <x:c r="C60" s="72"/>
       <x:c r="D60" s="21" t="s">
-        <x:v>130</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="E60" s="16" t="s">
-        <x:v>131</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="F60" s="75"/>
       <x:c r="G60" s="45"/>
@@ -2472,10 +2436,10 @@
       <x:c r="B61" s="91"/>
       <x:c r="C61" s="72"/>
       <x:c r="D61" s="21" t="s">
-        <x:v>132</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E61" s="4" t="s">
-        <x:v>133</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="F61" s="75"/>
       <x:c r="G61" s="45"/>
@@ -2486,10 +2450,10 @@
       <x:c r="B62" s="91"/>
       <x:c r="C62" s="72"/>
       <x:c r="D62" s="21" t="s">
-        <x:v>134</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E62" s="16" t="s">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F62" s="75"/>
       <x:c r="G62" s="45"/>
@@ -2500,10 +2464,10 @@
       <x:c r="B63" s="91"/>
       <x:c r="C63" s="72"/>
       <x:c r="D63" s="21" t="s">
-        <x:v>136</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="E63" s="16" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="F63" s="75"/>
       <x:c r="G63" s="45"/>
@@ -2514,10 +2478,10 @@
       <x:c r="B64" s="91"/>
       <x:c r="C64" s="72"/>
       <x:c r="D64" s="21" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="E64" s="16" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="F64" s="75"/>
       <x:c r="G64" s="45"/>
@@ -2528,10 +2492,10 @@
       <x:c r="B65" s="91"/>
       <x:c r="C65" s="72"/>
       <x:c r="D65" s="21" t="s">
-        <x:v>140</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="E65" s="16" t="s">
-        <x:v>141</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="F65" s="75"/>
       <x:c r="G65" s="45"/>
@@ -2542,10 +2506,10 @@
       <x:c r="B66" s="91"/>
       <x:c r="C66" s="72"/>
       <x:c r="D66" s="21" t="s">
-        <x:v>142</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="E66" s="16" t="s">
-        <x:v>143</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="F66" s="75"/>
       <x:c r="G66" s="45"/>
@@ -2556,10 +2520,10 @@
       <x:c r="B67" s="91"/>
       <x:c r="C67" s="72"/>
       <x:c r="D67" s="21" t="s">
-        <x:v>144</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="E67" s="16" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="F67" s="75"/>
       <x:c r="G67" s="45"/>
@@ -2570,10 +2534,10 @@
       <x:c r="B68" s="91"/>
       <x:c r="C68" s="72"/>
       <x:c r="D68" s="21" t="s">
-        <x:v>146</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="E68" s="16" t="s">
-        <x:v>147</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="F68" s="75"/>
       <x:c r="G68" s="45"/>
@@ -2584,10 +2548,10 @@
       <x:c r="B69" s="91"/>
       <x:c r="C69" s="72"/>
       <x:c r="D69" s="21" t="s">
-        <x:v>148</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="E69" s="16" t="s">
-        <x:v>149</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="F69" s="75"/>
       <x:c r="G69" s="45"/>
@@ -2598,10 +2562,10 @@
       <x:c r="B70" s="91"/>
       <x:c r="C70" s="72"/>
       <x:c r="D70" s="23" t="s">
-        <x:v>150</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="E70" s="16" t="s">
-        <x:v>151</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="F70" s="75"/>
       <x:c r="G70" s="45"/>
@@ -2612,10 +2576,10 @@
       <x:c r="B71" s="91"/>
       <x:c r="C71" s="72"/>
       <x:c r="D71" s="21" t="s">
-        <x:v>152</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E71" s="16" t="s">
-        <x:v>153</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="F71" s="75"/>
       <x:c r="G71" s="45"/>
@@ -2626,10 +2590,10 @@
       <x:c r="B72" s="91"/>
       <x:c r="C72" s="72"/>
       <x:c r="D72" s="21" t="s">
-        <x:v>154</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="E72" s="16" t="s">
-        <x:v>155</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="F72" s="75"/>
       <x:c r="G72" s="45"/>
@@ -2640,10 +2604,10 @@
       <x:c r="B73" s="91"/>
       <x:c r="C73" s="73"/>
       <x:c r="D73" s="21" t="s">
-        <x:v>156</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="E73" s="16" t="s">
-        <x:v>157</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="F73" s="75"/>
       <x:c r="G73" s="45"/>
@@ -2656,10 +2620,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="D74" s="21" t="s">
-        <x:v>158</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="E74" s="16" t="s">
-        <x:v>159</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="F74" s="75"/>
     </x:row>
@@ -2667,13 +2631,13 @@
       <x:c r="A75" s="77"/>
       <x:c r="B75" s="91"/>
       <x:c r="C75" s="50" t="s">
-        <x:v>160</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="D75" s="28" t="s">
-        <x:v>161</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="E75" s="18" t="s">
-        <x:v>162</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="F75" s="75"/>
     </x:row>
@@ -2681,13 +2645,13 @@
       <x:c r="A76" s="77"/>
       <x:c r="B76" s="91"/>
       <x:c r="C76" s="84" t="s">
-        <x:v>163</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="D76" s="29" t="s">
-        <x:v>164</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="E76" s="18" t="s">
-        <x:v>165</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="F76" s="75"/>
     </x:row>
@@ -2696,24 +2660,24 @@
       <x:c r="B77" s="91"/>
       <x:c r="C77" s="84"/>
       <x:c r="D77" s="29" t="s">
-        <x:v>166</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="E77" s="18" t="s">
-        <x:v>167</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="F77" s="75"/>
     </x:row>
     <x:row r="78" ht="16.5" customHeight="1">
       <x:c r="A78" s="77"/>
       <x:c r="B78" s="91"/>
-      <x:c r="C78" s="50" t="s">
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="D78" s="26" t="s">
-        <x:v>169</x:v>
+      <x:c r="C78" s="50" t="str">
+        <x:v>Maternal Mortality</x:v>
+      </x:c>
+      <x:c r="D78" s="26" t="str">
+        <x:v>Bangladesh Maternal Mortality Survey</x:v>
       </x:c>
       <x:c r="E78" s="18" t="s">
-        <x:v>170</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="F78" s="75"/>
     </x:row>
@@ -2721,41 +2685,41 @@
       <x:c r="A79" s="77"/>
       <x:c r="B79" s="91"/>
       <x:c r="C79" s="50" t="s">
-        <x:v>171</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="D79" s="30" t="s">
-        <x:v>172</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="E79" s="18" t="s">
-        <x:v>173</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="F79" s="75"/>
     </x:row>
     <x:row r="80" ht="16.5" customHeight="1">
       <x:c r="A80" s="77"/>
       <x:c r="B80" s="91"/>
-      <x:c r="C80" s="50" t="s">
-        <x:v>174</x:v>
+      <x:c r="C80" s="50" t="str">
+        <x:v>Infectious Disease</x:v>
       </x:c>
       <x:c r="D80" s="21" t="s">
-        <x:v>175</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="E80" s="18" t="s">
-        <x:v>176</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="F80" s="75"/>
     </x:row>
     <x:row r="81" ht="16.5" customHeight="1">
       <x:c r="A81" s="77"/>
       <x:c r="B81" s="91"/>
-      <x:c r="C81" s="50" t="s">
-        <x:v>177</x:v>
-      </x:c>
-      <x:c r="D81" s="26" t="s">
-        <x:v>178</x:v>
+      <x:c r="C81" s="50" t="str">
+        <x:v>Rohingya Health Bulletin</x:v>
+      </x:c>
+      <x:c r="D81" s="26" t="str">
+        <x:v>Rohingya Health Bulletin 2018</x:v>
       </x:c>
       <x:c r="E81" s="18" t="s">
-        <x:v>179</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F81" s="75"/>
     </x:row>
@@ -2763,13 +2727,13 @@
       <x:c r="A82" s="77"/>
       <x:c r="B82" s="91"/>
       <x:c r="C82" s="50" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="D82" s="26" t="s">
-        <x:v>181</x:v>
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="D82" s="26" t="str">
+        <x:v>eHealth August 2012</x:v>
       </x:c>
       <x:c r="E82" s="18" t="s">
-        <x:v>182</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="F82" s="75"/>
     </x:row>
@@ -2777,27 +2741,27 @@
       <x:c r="A83" s="77"/>
       <x:c r="B83" s="91"/>
       <x:c r="C83" s="50" t="s">
-        <x:v>183</x:v>
-      </x:c>
-      <x:c r="D83" s="26" t="s">
-        <x:v>184</x:v>
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="D83" s="26" t="str">
+        <x:v>Global Climate Change: Health Impacts on Bangladesh</x:v>
       </x:c>
       <x:c r="E83" s="18" t="s">
-        <x:v>185</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="F83" s="75"/>
     </x:row>
     <x:row r="84" ht="16.5" customHeight="1">
       <x:c r="A84" s="77"/>
       <x:c r="B84" s="91"/>
-      <x:c r="C84" s="88" t="s">
-        <x:v>186</x:v>
+      <x:c r="C84" s="88" t="str">
+        <x:v>Measles and Rubella Bulletin</x:v>
       </x:c>
       <x:c r="D84" s="21" t="s">
-        <x:v>187</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="E84" s="18" t="s">
-        <x:v>188</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="F84" s="75"/>
     </x:row>
@@ -2806,10 +2770,10 @@
       <x:c r="B85" s="91"/>
       <x:c r="C85" s="89"/>
       <x:c r="D85" s="21" t="s">
-        <x:v>189</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="E85" s="18" t="s">
-        <x:v>190</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="F85" s="75"/>
     </x:row>
@@ -2818,10 +2782,10 @@
       <x:c r="B86" s="91"/>
       <x:c r="C86" s="89"/>
       <x:c r="D86" s="26" t="s">
-        <x:v>191</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="E86" s="18" t="s">
-        <x:v>192</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="F86" s="75"/>
     </x:row>
@@ -2830,10 +2794,10 @@
       <x:c r="B87" s="91"/>
       <x:c r="C87" s="89"/>
       <x:c r="D87" s="26" t="s">
-        <x:v>193</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="E87" s="18" t="s">
-        <x:v>194</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="F87" s="75"/>
     </x:row>
@@ -2842,26 +2806,26 @@
       <x:c r="B88" s="91"/>
       <x:c r="C88" s="90"/>
       <x:c r="D88" s="26" t="s">
-        <x:v>195</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="E88" s="18" t="s">
-        <x:v>196</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="F88" s="75"/>
     </x:row>
     <x:row r="89" ht="28.5" customHeight="1">
       <x:c r="A89" s="77"/>
       <x:c r="B89" s="82" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="C89" s="58" t="s">
-        <x:v>198</x:v>
-      </x:c>
-      <x:c r="D89" s="61" t="s">
-        <x:v>199</x:v>
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="C89" s="58" t="str">
+        <x:v>National Institute of Cardiovascular Diseases</x:v>
+      </x:c>
+      <x:c r="D89" s="61" t="str">
+        <x:v>NICVD Cardiovascular Journal (Resource 40dbe_5098)</x:v>
       </x:c>
       <x:c r="E89" s="18" t="s">
-        <x:v>200</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="F89" s="75"/>
       <x:c r="G89" s="46"/>
@@ -2871,9 +2835,11 @@
       <x:c r="A90" s="77"/>
       <x:c r="B90" s="82"/>
       <x:c r="C90" s="59"/>
-      <x:c r="D90" s="62"/>
+      <x:c r="D90" s="62" t="str">
+        <x:v>NICVD Cardiovascular Journal (Resource 43724_24444)</x:v>
+      </x:c>
       <x:c r="E90" s="18" t="s">
-        <x:v>201</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="F90" s="75"/>
       <x:c r="G90" s="46"/>
@@ -2883,9 +2849,11 @@
       <x:c r="A91" s="77"/>
       <x:c r="B91" s="82"/>
       <x:c r="C91" s="59"/>
-      <x:c r="D91" s="62"/>
+      <x:c r="D91" s="62" t="str">
+        <x:v>NICVD Cardiovascular Journal (Resource 6dc7e_11451)</x:v>
+      </x:c>
       <x:c r="E91" s="18" t="s">
-        <x:v>202</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="F91" s="75"/>
       <x:c r="G91" s="46"/>
@@ -2895,9 +2863,11 @@
       <x:c r="A92" s="77"/>
       <x:c r="B92" s="85"/>
       <x:c r="C92" s="60"/>
-      <x:c r="D92" s="63"/>
+      <x:c r="D92" s="63" t="str">
+        <x:v>NICVD Cardiovascular Journal (Resource 32e70_4921)</x:v>
+      </x:c>
       <x:c r="E92" s="18" t="s">
-        <x:v>203</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="F92" s="75"/>
       <x:c r="G92" s="46"/>
@@ -2906,16 +2876,16 @@
     <x:row r="93" ht="15" customHeight="1">
       <x:c r="A93" s="77"/>
       <x:c r="B93" s="80" t="s">
-        <x:v>204</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="C93" s="78" t="s">
-        <x:v>205</x:v>
-      </x:c>
-      <x:c r="D93" s="27" t="s">
-        <x:v>206</x:v>
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="D93" s="27" t="str">
+        <x:v>Bangladesh Health Workforce Strategy 2024</x:v>
       </x:c>
       <x:c r="E93" s="18" t="s">
-        <x:v>207</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="F93" s="75"/>
       <x:c r="G93" s="45"/>
@@ -2926,10 +2896,10 @@
       <x:c r="B94" s="80"/>
       <x:c r="C94" s="79"/>
       <x:c r="D94" s="27" t="s">
-        <x:v>208</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="E94" s="18" t="s">
-        <x:v>209</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="F94" s="75"/>
       <x:c r="G94" s="45"/>
@@ -2940,10 +2910,10 @@
       <x:c r="B95" s="80"/>
       <x:c r="C95" s="79"/>
       <x:c r="D95" s="27" t="s">
-        <x:v>210</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="E95" s="18" t="s">
-        <x:v>211</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="F95" s="75"/>
       <x:c r="G95" s="45"/>
@@ -2954,10 +2924,10 @@
       <x:c r="B96" s="80"/>
       <x:c r="C96" s="79"/>
       <x:c r="D96" s="27" t="s">
-        <x:v>212</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="E96" s="18" t="s">
-        <x:v>213</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="F96" s="75"/>
       <x:c r="G96" s="45"/>
@@ -2968,10 +2938,10 @@
       <x:c r="B97" s="80"/>
       <x:c r="C97" s="79"/>
       <x:c r="D97" s="31" t="s">
-        <x:v>214</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="E97" s="18" t="s">
-        <x:v>215</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="F97" s="75"/>
       <x:c r="G97" s="45"/>
@@ -2982,10 +2952,10 @@
       <x:c r="B98" s="80"/>
       <x:c r="C98" s="79"/>
       <x:c r="D98" s="27" t="s">
-        <x:v>216</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="E98" s="18" t="s">
-        <x:v>217</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="F98" s="75"/>
       <x:c r="G98" s="45"/>
@@ -2996,10 +2966,10 @@
       <x:c r="B99" s="80"/>
       <x:c r="C99" s="79"/>
       <x:c r="D99" s="27" t="s">
-        <x:v>218</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="E99" s="18" t="s">
-        <x:v>219</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="F99" s="75"/>
       <x:c r="G99" s="45"/>
@@ -3010,10 +2980,10 @@
       <x:c r="B100" s="80"/>
       <x:c r="C100" s="79"/>
       <x:c r="D100" s="27" t="s">
-        <x:v>220</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="E100" s="18" t="s">
-        <x:v>221</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="F100" s="75"/>
       <x:c r="G100" s="45"/>
@@ -3024,10 +2994,10 @@
       <x:c r="B101" s="80"/>
       <x:c r="C101" s="79"/>
       <x:c r="D101" s="27" t="s">
-        <x:v>222</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="E101" s="18" t="s">
-        <x:v>223</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="F101" s="75"/>
       <x:c r="G101" s="45"/>
@@ -3036,16 +3006,16 @@
     <x:row r="102" ht="15.75" customHeight="1">
       <x:c r="A102" s="77"/>
       <x:c r="B102" s="86" t="s">
-        <x:v>224</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="C102" s="51" t="s">
-        <x:v>225</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="D102" s="33" t="s">
-        <x:v>226</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="E102" s="19" t="s">
-        <x:v>227</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="F102" s="75"/>
       <x:c r="G102" s="46"/>
@@ -3054,13 +3024,13 @@
       <x:c r="A103" s="77"/>
       <x:c r="B103" s="87"/>
       <x:c r="C103" s="51" t="s">
-        <x:v>228</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="D103" s="33" t="s">
-        <x:v>229</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="E103" s="18" t="s">
-        <x:v>230</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="F103" s="75"/>
       <x:c r="G103" s="46"/>
@@ -3068,16 +3038,16 @@
     <x:row r="104" ht="15" customHeight="1">
       <x:c r="A104" s="77"/>
       <x:c r="B104" s="57" t="s">
-        <x:v>231</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="C104" s="55" t="s">
-        <x:v>232</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="D104" s="33" t="s">
-        <x:v>233</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="E104" s="37" t="s">
-        <x:v>234</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="F104" s="75"/>
     </x:row>
@@ -3086,10 +3056,10 @@
       <x:c r="B105" s="57"/>
       <x:c r="C105" s="56"/>
       <x:c r="D105" s="33" t="s">
-        <x:v>235</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="E105" s="37" t="s">
-        <x:v>236</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F105" s="75"/>
       <x:c r="H105" s="41"/>
@@ -3143,10 +3113,10 @@
       <x:c r="B106" s="57"/>
       <x:c r="C106" s="56"/>
       <x:c r="D106" s="33" t="s">
-        <x:v>237</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="E106" s="37" t="s">
-        <x:v>238</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="F106" s="75"/>
       <x:c r="H106" s="41"/>
@@ -3200,10 +3170,10 @@
       <x:c r="B107" s="57"/>
       <x:c r="C107" s="56"/>
       <x:c r="D107" s="33" t="s">
-        <x:v>239</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="E107" s="37" t="s">
-        <x:v>240</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="F107" s="75"/>
       <x:c r="H107" s="41"/>
@@ -3257,10 +3227,10 @@
       <x:c r="B108" s="57"/>
       <x:c r="C108" s="56"/>
       <x:c r="D108" s="33" t="s">
-        <x:v>241</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="E108" s="37" t="s">
-        <x:v>242</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="F108" s="75"/>
       <x:c r="H108" s="41"/>
@@ -3314,10 +3284,10 @@
       <x:c r="B109" s="57"/>
       <x:c r="C109" s="56"/>
       <x:c r="D109" s="33" t="s">
-        <x:v>243</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="E109" s="37" t="s">
-        <x:v>244</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="F109" s="75"/>
       <x:c r="H109" s="41"/>
@@ -3371,10 +3341,10 @@
       <x:c r="B110" s="57"/>
       <x:c r="C110" s="56"/>
       <x:c r="D110" s="33" t="s">
-        <x:v>245</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="E110" s="37" t="s">
-        <x:v>246</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="F110" s="75"/>
       <x:c r="H110" s="41"/>
@@ -3428,10 +3398,10 @@
       <x:c r="B111" s="57"/>
       <x:c r="C111" s="56"/>
       <x:c r="D111" s="33" t="s">
-        <x:v>247</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="E111" s="37" t="s">
-        <x:v>248</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="F111" s="75"/>
       <x:c r="H111" s="41"/>
@@ -3485,10 +3455,10 @@
       <x:c r="B112" s="57"/>
       <x:c r="C112" s="56"/>
       <x:c r="D112" s="34" t="s">
-        <x:v>249</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="E112" s="37" t="s">
-        <x:v>250</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="F112" s="75"/>
       <x:c r="H112" s="41"/>
@@ -3542,10 +3512,10 @@
       <x:c r="B113" s="57"/>
       <x:c r="C113" s="56"/>
       <x:c r="D113" s="35" t="s">
-        <x:v>251</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="E113" s="38" t="s">
-        <x:v>252</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="F113" s="76"/>
       <x:c r="H113" s="41"/>
@@ -3947,121 +3917,121 @@
     <x:mergeCell ref="C46:C73"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="R134caf29bb3d4377"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="R3eec689893804f00"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="R3f61182304fe4768"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="Ra38a681c49534379"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="R2b1a74d6bc464e7d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="R8b3d870a8e174306"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="R4509be953eab4586"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="R5f35b21d3b304887"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="Rf2f5345afa2b46c3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="Re208369d06394e2e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="R55768a70f40944fa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="R59d90803c76c4178"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="R9eaa3cb8ebe64be7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="Raa8af87e911847c3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="Rddfaece3c0d04f7f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="R7859c404d4a74ed2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="Rd4288d7c334542a3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="R6fa69b0cc2a8484e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="R80de0637f58e427e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="R523d343e14524e13"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="R18b4059af93049a2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="R7cff4c608fb34d19"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="R1ae24a86e83a41f8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="Rcf9709d8072b4089"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="R21e19fb343754a28"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="Rae3c57129da14355"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="Rf3fb70f07c4245d6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="R44525a9679954621"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="Rc5e533245a794131"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="Rf75c5f1caa574c7c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="R2b5b0604248847cc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="R53d7d46ecc7e43e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R10926df0ba7d4c27"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="R8f10dee7d2c14287"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="R27c2423b4f1541bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="R028a44e38e584812"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="Rb0e691f4cc3b41ea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="R8f23742de8004e93"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R8f496140c0444c13"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R00fcbda17a3b4ed4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="R8383b4704f254f25"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="Rfa2110b449d44fdc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Raa5310d1db6747c3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="Rf9e8da0c4f754ba2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="R6e38084bd33a4915"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="R2feb18646ea74c07"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="R0dc0ff68aa124fe0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="R5d3c6af831a54f67"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="R9b563b8d65674de0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="Rf59301754dab48d0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R7d21f391c8444ed3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="Red8968d938b64cb3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="R3fc59f5623fd4600"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="R4b27fd9dbbae47a2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="Rc95dc2f865ca438e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="Rfaa8c17410e74c12"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R3976f9adf6e34348"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="R80e8cf2462bf4fae"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="R14f41827dc65425d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="R8cfca85de9fe49d9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="R9f120992403541d1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R9a0a25df79414695"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R05b27db3ae2a424e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="R44b8800581d84701"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="Rc63d776d2bf145dc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R0d3f0e5197694bb0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="Rd158a0890ea2412f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="R93437fe83fbf4453"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="Ra8c1afdcc3754a83"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="Ra9badb1d0a4f4fb6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="Rae63746aea324c9f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="R856df7cb9ab04b67"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="R424e5b94209c4a68"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="Ra1b0405776384e59"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="R3d1ca8aeade2427c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="R5783ed290c0a47bd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="Rbb0f0f373a7b4588"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="R5231c36c0fd34ff4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="Ra5d12da25aa54937"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="Rfb71254d29744d1e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="Rcd09bb75652341a3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="Rbc2d982eba5c428e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="Ra0a1ca5f3606458c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="R4d364f72d4354156"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="R392ecf656e334710"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="R4472aa94850a4076"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="Raae7b97b746149e9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="R5912c868210e46d1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="R9e9e82bfee4247cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="R570b635fbf4e40d5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="Raba6a021ca534b56"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="R48aa918e3d684bec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="R53e761b19d1b44e8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="Re9840a83804f43dd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="Ra29ebc5c309d4366"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="R185b288c5e8a4021"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="R50e1af5254934e64"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="Rac26eae02c3b4c94"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="Rb5b808896b664715"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="R011a2ca01aae41a9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="R10817c597f7f4c97"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="R95a87f32e37c44e4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="Rc1be0388a4194bc3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="R4fac923dc54c4e6c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="Rd96ae88cb3304743"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="Rb72fe2469a664aa8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="R9a9c922a6c2f4b40"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="R2e787d516c0e43e5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="R125691a2c42b4e04"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="Rcef58b2af86c463b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="Rba97bc8c0e6747cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="R7d234d0b6b2b4fa8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="Rf6bbc43a6b8349f9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="R515564bb153a4f68"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="Rbf23fbb517fb44c3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="Rbeccb4b23a094dfc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="Recd29fb5bcff4473"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="Re4760e25314d47a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="R47b5bcee4f26418f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="R766c4be5a04f4b39"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="Rc41f266aefd64888"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="R824c8da93eed43c3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="R068e1c6e2f134b3c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="R38e567398ff847ac"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="R8cd07b5076a54885"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="R6d55602b845d46ba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="Rbc4d76d0aa11407c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="R9c5008a712134423"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="R1c4bb286585e4804"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R9af7329389214341"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="Rd5da895853394d37"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="R1b0459a7e5704ab7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="R3fa49c797d1741fa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="Rdb24413c8f534ab4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="R8710f308218a4866"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="Rbb4a80965f514095"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="R16d6365f65f34239"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="Re3f834cfefda4394"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="Rf8519e8529094a6e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="Rb4f56c5825294076"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="R987d38bfe2ad4b85"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="Rf631302d07334e05"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="Rca4ac825dfe14a4b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="Rb3e17aa9812247f6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="Reab833975a1f461a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="R32287cbc28b444d8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="R5e11953dbe234bf8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="Rff6dac1c51db410a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="Ra69a6e311300418e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="R76f2b2c7380b42da"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="R12463fdce797450b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="Rebcd6e351d6e4e3f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="R6c6f42f614de4dab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R856b4f6a5ded4dd4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rc9c81b1727174011"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="R71ea3d9017af4812"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="R2b5e7dcac07847ce"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="R1ebde5c8a88040c1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="R0718bb74f67c46ba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="Rdff23569a59d4dcb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="R077cbd75dad6410c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="R93b4914a7c754b01"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="Rdf54d6fb568a4db1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="Re18c859b7db9423b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="R8da5b551071f44ab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R454567e1423e4993"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R6e4d48cd0fd94572"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="R48044ddf38dd4c56"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="R18e89259439040c3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="Rdf61926f410f493e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="R0dd28fde376a4587"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R9e2a194596c34bbc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="Re1012ecc6ca54d8b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="Rb4b564ec402a418c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="R94d1ebb0feb84986"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="Ra3c6dfa943ef42c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R0edcfb8475ed44a2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R75d8f34f3cd14bc3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="Ra34d06d3099d4ada"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="Re88b01b4a76c4fe5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R3418764e7fcb4ae9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="Rfc11f7b17c684c96"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="Rc0a1ca2c1259473f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="Rfa8e53c2d9d14370"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="R0e19c6082d7c4a1c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="R1e3c4494e0f54b81"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="Rc540299ad3c34ec4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="Radc7efa81d524152"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="R01cfc73248614453"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="R8c0e38dcbb9449bd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="R3b4aea83e989461f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="R13d17389f7064d93"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="Rd8ad225e2d624fa2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="R9e8804ac84bc450c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="R12577b58cf99492d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="R710a0fb50d9a47ec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="Rc257ca7ea56948a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="Re32ab12d87284895"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="R67fc789c50734a48"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="R5d3fadf402724a24"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="R8aff58307607456f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="Re94481e0315348dd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="R7e24624127c44db3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="R2e2a0b312faa4043"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="R5c086cbebef24617"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="R1f88bac37ac14977"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="R89929becba63477f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="Rdcfc7bc89aed4b50"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="Re2662a6bcd984022"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="R63647ff02e49449a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="R528e84242f1a40a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="Ra22f8b5b66e345b2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="R16bd4dc835aa4517"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="Rbcfe06df07654fa7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="Rd5000c7a68874594"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="R483e46f67a1440de"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="Rd1895999d73d4b5f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="R64c3b95963404be1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="R0ec5dee00b8643f7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="R96be9953635e477d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="R4f4dcab7b2254482"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="Rc88e510ee4cb4a8d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="R9d5fe8e9d7b04e55"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="R69f2299b93db4c4d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="Ra6117f56a7ef4f11"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="Rb641b67587834f6c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="R0e967800b1aa46b7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="R93ae229a92a547fe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="R7919573db9ed4a10"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="Ra5da7263f01c4c6d"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4667,7 +4637,7 @@
         <x:v>Mental Health</x:v>
       </x:c>
       <x:c r="E23" s="108" t="str">
-        <x:v>Preventation and Management of Mental Health Conditions in Bangladesh</x:v>
+        <x:v>Prevention and Management of Mental Health Conditions in Bangladesh</x:v>
       </x:c>
       <x:c r="F23" s="110" t="str">
         <x:v>https://cdn.who.int/media/docs/default-source/mental-health/special-initiative/mhic-bangladesh-report-25.07.25v2.pdf?sfvrsn=7f87a3c6_3</x:v>
@@ -4693,7 +4663,7 @@
         <x:v>Maternal Health</x:v>
       </x:c>
       <x:c r="E24" s="108" t="str">
-        <x:v>United Nations Populations fund</x:v>
+        <x:v>UNFPA Country Programme Document for Bangladesh 2022-2026</x:v>
       </x:c>
       <x:c r="F24" s="110" t="str">
         <x:v>https://www.unfpa.org/sites/default/files/portal-document/ENG_DP.FPA_.CPD_.BGD_.10%20-%20Bangladesh%20CPD%20-%20FINAL%20-%2018Jul21.pdf</x:v>
@@ -4719,7 +4689,7 @@
         <x:v>Maternal Health</x:v>
       </x:c>
       <x:c r="E25" s="108" t="str">
-        <x:v>United Nations Populations fund</x:v>
+        <x:v>UNFPA Country Programme Document for Bangladesh 2017-2020</x:v>
       </x:c>
       <x:c r="F25" s="110" t="str">
         <x:v>https://www.unfpa.org/sites/default/files/portal-document/N1620634.pdf</x:v>
@@ -4745,7 +4715,7 @@
         <x:v>Maternal Health</x:v>
       </x:c>
       <x:c r="E26" s="108" t="str">
-        <x:v>United Nations Populations fund</x:v>
+        <x:v>UNDAF Action Plan Bangladesh 2012-2016</x:v>
       </x:c>
       <x:c r="F26" s="110" t="str">
         <x:v>https://www.unfpa.org/sites/default/files/portal-document/Bangladesh_UNDAF%202012-2016.pdf.pdf</x:v>
@@ -4771,7 +4741,7 @@
         <x:v>Maternal Health</x:v>
       </x:c>
       <x:c r="E27" s="108" t="str">
-        <x:v>United Nations Populations fund</x:v>
+        <x:v>UNFPA Final Country Programme Document for Bangladesh 2012-2016</x:v>
       </x:c>
       <x:c r="F27" s="110" t="str">
         <x:v>https://www.unfpa.org/sites/default/files/portal-document/Bangladesh_CPD%202012-2016.pdf.pdf</x:v>
@@ -6094,10 +6064,10 @@
         <x:v>DGHS</x:v>
       </x:c>
       <x:c r="D78" s="108" t="str">
-        <x:v>Maternal Morality</x:v>
+        <x:v>Maternal Mortality</x:v>
       </x:c>
       <x:c r="E78" s="108" t="str">
-        <x:v>Bangladesh Maternal Morality Servey</x:v>
+        <x:v>Bangladesh Maternal Mortality Survey</x:v>
       </x:c>
       <x:c r="F78" s="110" t="str">
         <x:v>https://old.dghs.gov.bd/licts_file/images/BMMS/BMMS_2010_color.pdf</x:v>
@@ -6120,7 +6090,7 @@
         <x:v>DGHS</x:v>
       </x:c>
       <x:c r="D79" s="108" t="str">
-        <x:v>Infectious Diesease</x:v>
+        <x:v>Infectious Disease</x:v>
       </x:c>
       <x:c r="E79" s="108" t="str">
         <x:v>Mapping of the Infectious Disease Surveillance System in Bangladesh</x:v>
@@ -6172,10 +6142,10 @@
         <x:v>DGHS</x:v>
       </x:c>
       <x:c r="D81" s="108" t="str">
-        <x:v>Rohinga Heath Bulletin</x:v>
+        <x:v>Rohingya Health Bulletin</x:v>
       </x:c>
       <x:c r="E81" s="108" t="str">
-        <x:v>Rohinga Health Bulletin 2018</x:v>
+        <x:v>Rohingya Health Bulletin 2018</x:v>
       </x:c>
       <x:c r="F81" s="110" t="str">
         <x:v>https://old.dghs.gov.bd/images/docs/Publicaations/HB_030718.pdf</x:v>
@@ -6201,7 +6171,7 @@
         <x:v>E-Health</x:v>
       </x:c>
       <x:c r="E82" s="108" t="str">
-        <x:v>eHealth Auguest 2012</x:v>
+        <x:v>eHealth August 2012</x:v>
       </x:c>
       <x:c r="F82" s="110" t="str">
         <x:v>https://old.dghs.gov.bd/licts_file/images/eHealth/our_eHealth_Aug_2012.pdf</x:v>
@@ -6227,7 +6197,7 @@
         <x:v>Climate</x:v>
       </x:c>
       <x:c r="E83" s="108" t="str">
-        <x:v>বাংলাদেশের স্বাস্থ্য খাতে জল-বায়ু পরিবর্তনের প্রভাব (২০০৯ সালে কোপেনহেগেন কপ ১৫ উপলক্ষে প্রস্তুতকৃত)</x:v>
+        <x:v>Global Climate Change: Health Impacts on Bangladesh</x:v>
       </x:c>
       <x:c r="F83" s="110" t="str">
         <x:v>https://old.dghs.gov.bd/licts_file/images/Climate_Change/2009_ClimateChange2009.pdf</x:v>
@@ -6250,7 +6220,7 @@
         <x:v>DGHS</x:v>
       </x:c>
       <x:c r="D84" s="108" t="str">
-        <x:v>Measles and Rebella Bulletin</x:v>
+        <x:v>Measles and Rubella Bulletin</x:v>
       </x:c>
       <x:c r="E84" s="108" t="str">
         <x:v>MR bulletin ( 2nd quarter 2021)</x:v>
@@ -6276,7 +6246,7 @@
         <x:v>DGHS</x:v>
       </x:c>
       <x:c r="D85" s="108" t="str">
-        <x:v>Measles and Rebella Bulletin</x:v>
+        <x:v>Measles and Rubella Bulletin</x:v>
       </x:c>
       <x:c r="E85" s="108" t="str">
         <x:v>MR Bulletin Volume 1</x:v>
@@ -6302,7 +6272,7 @@
         <x:v>DGHS</x:v>
       </x:c>
       <x:c r="D86" s="108" t="str">
-        <x:v>Measles and Rebella Bulletin</x:v>
+        <x:v>Measles and Rubella Bulletin</x:v>
       </x:c>
       <x:c r="E86" s="108" t="str">
         <x:v>MR Bulletin Volume 2</x:v>
@@ -6328,7 +6298,7 @@
         <x:v>DGHS</x:v>
       </x:c>
       <x:c r="D87" s="108" t="str">
-        <x:v>Measles and Rebella Bulletin</x:v>
+        <x:v>Measles and Rubella Bulletin</x:v>
       </x:c>
       <x:c r="E87" s="108" t="str">
         <x:v>MR Bulletin Volume 3</x:v>
@@ -6354,7 +6324,7 @@
         <x:v>DGHS</x:v>
       </x:c>
       <x:c r="D88" s="108" t="str">
-        <x:v>Measles and Rebella Bulletin</x:v>
+        <x:v>Measles and Rubella Bulletin</x:v>
       </x:c>
       <x:c r="E88" s="108" t="str">
         <x:v>Measles Update(Till 14/05/26)</x:v>
@@ -6380,10 +6350,10 @@
         <x:v>NICVD</x:v>
       </x:c>
       <x:c r="D89" s="108" t="str">
-        <x:v>National Institute of cardiovascular Disease</x:v>
+        <x:v>National Institute of Cardiovascular Diseases</x:v>
       </x:c>
       <x:c r="E89" s="108" t="str">
-        <x:v>Cardiovascular Diseases  Information</x:v>
+        <x:v>NICVD Cardiovascular Journal (Resource 40dbe_5098)</x:v>
       </x:c>
       <x:c r="F89" s="110" t="str">
         <x:v>https://pub.flowpaper.com/docs/https:/www.nicvd.gov.bd/uploadFile/journal/40dbe_5098.pdf</x:v>
@@ -6406,10 +6376,10 @@
         <x:v>NICVD</x:v>
       </x:c>
       <x:c r="D90" s="108" t="str">
-        <x:v>National Institute of cardiovascular Disease</x:v>
+        <x:v>National Institute of Cardiovascular Diseases</x:v>
       </x:c>
       <x:c r="E90" s="108" t="str">
-        <x:v>Cardiovascular Diseases  Information</x:v>
+        <x:v>NICVD Cardiovascular Journal (Resource 43724_24444)</x:v>
       </x:c>
       <x:c r="F90" s="110" t="str">
         <x:v>https://pub.flowpaper.com/docs/https:/www.nicvd.gov.bd/uploadFile/journal/43724_24444.pdf</x:v>
@@ -6432,10 +6402,10 @@
         <x:v>NICVD</x:v>
       </x:c>
       <x:c r="D91" s="108" t="str">
-        <x:v>National Institute of cardiovascular Disease</x:v>
+        <x:v>National Institute of Cardiovascular Diseases</x:v>
       </x:c>
       <x:c r="E91" s="108" t="str">
-        <x:v>Cardiovascular Diseases  Information</x:v>
+        <x:v>NICVD Cardiovascular Journal (Resource 6dc7e_11451)</x:v>
       </x:c>
       <x:c r="F91" s="110" t="str">
         <x:v>https://pub.flowpaper.com/docs/https:/www.nicvd.gov.bd/uploadFile/journal/6dc7e_11451.pdf</x:v>
@@ -6458,10 +6428,10 @@
         <x:v>NICVD</x:v>
       </x:c>
       <x:c r="D92" s="108" t="str">
-        <x:v>National Institute of cardiovascular Disease</x:v>
+        <x:v>National Institute of Cardiovascular Diseases</x:v>
       </x:c>
       <x:c r="E92" s="108" t="str">
-        <x:v>Cardiovascular Diseases  Information</x:v>
+        <x:v>NICVD Cardiovascular Journal (Resource 32e70_4921)</x:v>
       </x:c>
       <x:c r="F92" s="110" t="str">
         <x:v>https://pub.flowpaper.com/docs/https:/www.nicvd.gov.bd/uploadFile/journal/32e70_4921.pdf</x:v>
@@ -6487,7 +6457,7 @@
         <x:v>Policy and Administration</x:v>
       </x:c>
       <x:c r="E93" s="108" t="str">
-        <x:v>বাংলাদেশ হেলথ ওয়ার্কফোর্স স্ট্রাটেজি ২০২৪</x:v>
+        <x:v>Bangladesh Health Workforce Strategy 2024</x:v>
       </x:c>
       <x:c r="F93" s="110" t="str">
         <x:v>https://objectstorage.ap-dcc-gazipur-1.oraclecloud15.com/n/axvjbnqprylg/b/V2Ministry/o/office-hsd/2024/12/ab1c3ee0b4a54a69a4e3044865b01e23.pdf</x:v>
@@ -7152,7 +7122,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54f1c8c698ef491b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd09e8079c39a46bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>